<commit_message>
fix: resolve CGPA extraction with en-dash/hyphen separators and embed original resume modal viewer
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -670,10 +670,8 @@
       <c r="L2" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M2" s="2" t="n">
+        <v>9.279999999999999</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -2808,10 +2806,8 @@
       <c r="L25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M25" s="2" t="n">
+        <v>7.55</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
@@ -2996,10 +2992,8 @@
       <c r="L27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M27" s="2" t="n">
+        <v>9.710000000000001</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
@@ -3276,10 +3270,8 @@
       <c r="L30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M30" s="2" t="n">
+        <v>8.720000000000001</v>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
@@ -3370,10 +3362,8 @@
       <c r="L31" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M31" s="2" t="n">
+        <v>8.43</v>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
@@ -3652,10 +3642,8 @@
       <c r="L34" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M34" s="2" t="n">
+        <v>8.15</v>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: distinct LLM narratives, blank-start dashboard, strict CGPA dial
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -478,7 +478,7 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -690,10 +690,10 @@
         <v>35</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="T2" s="3" t="n">
         <v>0</v>
@@ -711,7 +711,7 @@
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>V Sree Raghu Vardhan qualifies as an eligible candidate with a total score of 94.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, Django, PostgreSQL, Redis. GitHub enrichment indicates: Veteran Builder (4.2 yrs on GitHub, 35 repos, 0 recent commits). 3 relevant Python/AI repositories identified. Primary area for review: No significant technical weaknesses observed. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 94.5/100, V Sree Raghu Vardhan stands out through cloud infrastructure (aws/azure), complemented by full stack capability (react/next.js/typescript). Plus strong public github footprint (veteran builder) rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, Redis maps to AI 37.0 and Python 30.0 bands. GitHub profile: Veteran Builder (4.2 yrs on GitHub, 35 repos [24 original], 45 contributions in past year [0 commits]). 3 relevant Python/AI repositories identified. Growth edge to probe in interview: polishing production hardening.</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 73490 41840</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>88.5</v>
+        <v>91</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>32</v>
@@ -757,7 +757,7 @@
         <v>14</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="L3" s="3" t="n">
         <v>5</v>
@@ -784,19 +784,19 @@
         <v>18</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="T3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="V3" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>Prathamesh Patil qualifies as an eligible candidate with a total score of 88.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, PostgreSQL, Redis, Docker. GitHub enrichment indicates: Veteran Builder (3.9 yrs on GitHub, 18 repos, 0 recent commits). 0 relevant Python/AI repositories identified. Primary area for review: No significant technical weaknesses observed. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Prathamesh Patil scored 91.0/100 (AI 32.0/40, Python 30.0/30, Cloud 14.0/15, GitHub 10.0/10), led by strong public github footprint (veteran builder) and automated testing / ci/cd pipeline Backed by distributed task queues (celery/rabbitmq/kafka). Stack centers on Python, FastAPI, PostgreSQL, Redis. GitHub: Veteran Builder (3.9 yrs on GitHub, 18 repos [17 original], 121 contributions in past year [0 commits, 28 PRs], 3 stars). 14 relevant Python/AI repositories identified. Watch-item: polishing production hardening. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -815,22 +815,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Sumaiya Sultana Shaik</t>
+          <t>Gourab Das</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>sultanasumaiya623@gmail.com</t>
+          <t>gourabdas1307@gmail.com</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91-7002572852</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>candidate_28.pdf</t>
+          <t>candidate_17.pdf</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>82.5</v>
+        <v>81.5</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>10</v>
@@ -856,8 +856,10 @@
       <c r="L4" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>7.1</v>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -866,20 +868,20 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Active Builder</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>2.7</v>
+        <v>6.3</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T4" s="3" t="n">
         <v>0</v>
@@ -892,12 +894,12 @@
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Docker, GCP, LangChain, LangGraph, RAG, React, Typescript, Graphql, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, Django, Flask, PostgreSQL, Redis, Docker, AWS, LangChain, LangGraph, RAG, React, Kafka, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java, Spring Boot</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Sumaiya Sultana Shaik qualifies as an eligible candidate with a total score of 82.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, PostgreSQL, Docker, GCP. GitHub enrichment indicates: Active Builder (2.7 yrs on GitHub, 29 repos, 0 recent commits). 14 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Gourab Das (81.5/100) impressed with advanced rag with hybrid search and reranking alongside async fastapi backend architecture. Also notable: postgresql with orm / schema migrations. Depth spans Python, FastAPI, Django, Flask, PostgreSQL, Redis (cloud 14.0/15, GitHub 10.0/10). Activity: Veteran Builder (6.3 yrs on GitHub, 21 repos [12 original], 3 contributions in past year [0 commits]). 4 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -907,22 +909,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Arjun Kumar</t>
+          <t>Vaibhav Wakde</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>roy.prajapat.143@gmail.com</t>
+          <t>vaibhavwakde266@gmail.com</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>+91-6396303191</t>
+          <t>+91-9307600143</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>candidate_08.pdf</t>
+          <t>candidate_33.pdf</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -931,16 +933,16 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>81.5</v>
+        <v>75.5</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>10</v>
@@ -948,8 +950,10 @@
       <c r="L5" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M5" s="2" t="n">
-        <v>8.279999999999999</v>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -962,16 +966,16 @@
         </is>
       </c>
       <c r="P5" s="3" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="T5" s="3" t="n">
         <v>0</v>
@@ -984,12 +988,12 @@
       </c>
       <c r="W5" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, PostgreSQL, AWS, LangChain, LangGraph, RAG, Embeddings, Gemini, Tensorflow, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, Flask, Docker, AWS, LangChain, LangGraph, LlamaIndex, RAG, ChromaDB, Weaviate, Tool Calling, Openai, Ollama, Transformers, Javascript, Pytest, GIT, SQL</t>
         </is>
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>Arjun Kumar qualifies as an eligible candidate with a total score of 81.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, Django, PostgreSQL, AWS. GitHub enrichment indicates: Veteran Builder (3.0 yrs on GitHub, 26 repos, 0 recent commits). 13 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Vaibhav Wakde (75.5/100) impressed with cloud infrastructure (aws/azure) alongside strong public github footprint (veteran builder). Also notable: automated testing / ci/cd pipeline. Depth spans Python, FastAPI, Flask, Docker, AWS, LangChain (cloud 10.0/15, GitHub 10.0/10). Activity: Veteran Builder (3.5 yrs on GitHub, 10 repos [10 original], 12 contributions in past year [0 commits]). 4 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -999,22 +1003,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Gourab Das</t>
+          <t>Arunima Saha</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>gourabdas1307@gmail.com</t>
+          <t>arunimasaha11@gmail.com</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>+91-7002572852</t>
+          <t>+91 9187656193</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>candidate_17.pdf</t>
+          <t>candidate_43.pdf</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1023,43 +1027,41 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>81.5</v>
+        <v>75.5</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Unlinked / Missing</t>
         </is>
       </c>
       <c r="P6" s="3" t="n">
-        <v>6.3</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
@@ -1078,12 +1080,12 @@
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, Flask, PostgreSQL, Redis, Docker, AWS, LangChain, LangGraph, RAG, React, Kafka, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java, Spring Boot</t>
+          <t>Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS, LangChain, LangGraph, RAG, Pinecone, Embeddings, Vector Search, Tool Calling, Openai, Gemini, Transformers, Rest Api, GIT, SQL</t>
         </is>
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>Gourab Das qualifies as an eligible candidate with a total score of 81.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), advanced rag with hybrid search and reranking, supported by core stack competencies in Python, FastAPI, Django, Flask, PostgreSQL. GitHub enrichment indicates: Veteran Builder (6.3 yrs on GitHub, 21 repos, 0 recent commits). 4 relevant Python/AI repositories identified. Primary area for review: No significant technical weaknesses observed. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Arunima Saha (75.5/100) impressed with advanced rag with hybrid search and reranking alongside ai evaluation pipeline (ragas/langsmith/trulens). Also notable: modern python backend framework (fastapi/django). Depth spans Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS (cloud 11.0/15, GitHub 0.0/10). Activity: No public GitHub profile provided. Interview focus should be no explicit testing (pytest/unit tests) mentioned, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1095,22 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Yash Maini</t>
+          <t>Abhinav Mishra</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>mainiyash2@gmail.com</t>
+          <t>abhinavmishra3322@gmail.com</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>+91-8920028757</t>
+          <t>+91 7701956829</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>candidate_13.pdf</t>
+          <t>candidate_10.pdf</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1117,25 +1119,27 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>73.5</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>10</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>8.609999999999999</v>
+        <v>3.5</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -1148,34 +1152,34 @@
         </is>
       </c>
       <c r="P7" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>0</v>
+        <v>4315</v>
       </c>
       <c r="T7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, GCP, AWS, LangChain, LangGraph, RAG, Faiss, Pinecone, Embeddings, Tool Calling, Openai, Claude, Pytorch, Tensorflow, Rest Api, Ci/Cd, SQL, Mongodb</t>
+          <t>Python, FastAPI, PostgreSQL, Redis, Azure, LangGraph, RAG, Openai, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd</t>
         </is>
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>Yash Maini qualifies as an eligible candidate with a total score of 78.0/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, Flask, PostgreSQL, Postgres. GitHub enrichment indicates: Veteran Builder (3.8 yrs on GitHub, 47 repos, 0 recent commits). 22 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Abhinav’s 3.4-year GitHub tenure reveals a veteran builder with 28 original repositories, proving sustained commitment beyond typical intern portfolios. His technical depth shines through stateful multi-agent orchestration using LangGraph and robust RAG pipelines, anchored by a modern FastAPI and PostgreSQL backend. The cloud_fullstack score indicates a minor gap in enterprise Azure deployment, though his Python and Redis proficiency mitigates this. This blend of architectural maturity and practical AI implementation makes him an immediate, low-risk asset for our engineering team.</t>
         </is>
       </c>
     </row>
@@ -1185,22 +1189,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Vaibhav Wakde</t>
+          <t>Hari Shanker Sharma</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>vaibhavwakde266@gmail.com</t>
+          <t>harishankersharma648@gmail.com</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>+91-9307600143</t>
+          <t>+91 8801109700</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>candidate_33.pdf</t>
+          <t>candidate_41.pdf</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -1209,19 +1213,19 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>75.5</v>
+        <v>73.5</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>3.5</v>
@@ -1238,14 +1242,14 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P8" s="3" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>0</v>
@@ -1264,12 +1268,12 @@
       </c>
       <c r="W8" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, Docker, AWS, LangChain, LangGraph, LlamaIndex, RAG, ChromaDB, Weaviate, Tool Calling, Openai, Ollama, Transformers, Javascript, Pytest, GIT, SQL</t>
+          <t>Python, FastAPI, PostgreSQL, Redis, Docker, Kubernetes, AWS, LangChain, LangGraph, RAG, Qdrant, Embeddings, Vector Search, Openai, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>Vaibhav Wakde qualifies as an eligible candidate with a total score of 75.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, Flask, Docker, AWS. GitHub enrichment indicates: Veteran Builder (3.5 yrs on GitHub, 10 repos, 0 recent commits). 4 relevant Python/AI repositories identified. Primary area for review: No significant technical weaknesses observed. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Hari Shanker Sharma scored 73.5/100 (AI 29.0/40, Python 27.0/30, Cloud 14.0/15, GitHub 0.0/10), led by distributed task queues (celery/rabbitmq/kafka) and stateful multi-agent orchestration (langgraph/crewai/autogen) Backed by vector database retrieval (chromadb/faiss/pinecone/qdrant). Stack centers on Python, FastAPI, PostgreSQL, Redis. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: low or dormant public github activity. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -1279,22 +1283,22 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Arunima Saha</t>
+          <t>Sumaiya Sultana Shaik</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>arunimasaha11@gmail.com</t>
+          <t>sultanasumaiya623@gmail.com</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>+91 9187656193</t>
+          <t>+91 97015 28467</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>candidate_43.pdf</t>
+          <t>candidate_28.pdf</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1303,34 +1307,34 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>75.5</v>
+        <v>72.5</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>23</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Unlinked / Missing</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P9" s="3" t="n">
@@ -1356,12 +1360,12 @@
       </c>
       <c r="W9" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS, LangChain, LangGraph, RAG, Pinecone, Embeddings, Vector Search, Tool Calling, Openai, Gemini, Transformers, Rest Api, GIT, SQL</t>
+          <t>Python, FastAPI, PostgreSQL, Docker, GCP, LangChain, LangGraph, RAG, React, Typescript, Graphql, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>Arunima Saha qualifies as an eligible candidate with a total score of 75.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), advanced rag with hybrid search and reranking, supported by core stack competencies in Python, FastAPI, PostgreSQL, Docker, Google Cloud. GitHub enrichment indicates: No public GitHub profile provided. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Sumaiya Sultana Shaik demonstrates promising architectural instincts through stateful multi-agent orchestration using LangGraph and CrewAI, paired with a solid FastAPI and PostgreSQL backend. Her experience integrating RAG pipelines with Docker and GCP shows practical fullstack capability. However, her public GitHub activity is currently dormant or inaccessible due to API limits, obscuring her broader engineering depth. The primary gap is a lack of evidence for Redis caching or performance optimization. Despite these unknowns, her core AI backend skills align well with our intern needs, warranting a technical interview to validate her hands-on proficiency.</t>
         </is>
       </c>
     </row>
@@ -1371,22 +1375,22 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Abhinav Mishra</t>
+          <t>Arjun Kumar</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>abhinavmishra3322@gmail.com</t>
+          <t>roy.prajapat.143@gmail.com</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>+91 7701956829</t>
+          <t>+91-6396303191</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>candidate_10.pdf</t>
+          <t>candidate_08.pdf</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1395,10 +1399,10 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>73.5</v>
+        <v>71.5</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>25</v>
@@ -1407,15 +1411,13 @@
         <v>8</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M10" s="2" t="n">
+        <v>8.279999999999999</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1424,14 +1426,14 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P10" s="3" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>0</v>
@@ -1450,12 +1452,12 @@
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Redis, Azure, LangGraph, RAG, Openai, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd</t>
+          <t>Python, FastAPI, Django, PostgreSQL, AWS, LangChain, LangGraph, RAG, Embeddings, Gemini, Tensorflow, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>Abhinav Mishra qualifies as an eligible candidate with a total score of 73.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, PostgreSQL, Redis, Azure. GitHub enrichment indicates: Veteran Builder (3.4 yrs on GitHub, 61 repos, 0 recent commits). 9 relevant Python/AI repositories identified. Primary area for review: No significant technical weaknesses observed. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 71.5/100, Arjun Kumar stands out through automated testing / ci/cd pipeline, complemented by observability and concurrency handling. Plus stateful multi-agent orchestration (langgraph/crewai/autogen) rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, AWS maps to AI 35.0 and Python 25.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -1465,22 +1467,22 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Hari Shanker Sharma</t>
+          <t>Kiran Naregal</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>harishankersharma648@gmail.com</t>
+          <t>kirnaregal7@gmail.com</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>+91 8801109700</t>
+          <t>9964923041</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>candidate_41.pdf</t>
+          <t>candidate_47.pdf</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1489,13 +1491,13 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>73.5</v>
+        <v>70.5</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>14</v>
@@ -1504,12 +1506,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>8.76</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Redis, Docker, Kubernetes, AWS, LangChain, LangGraph, RAG, Qdrant, Embeddings, Vector Search, Openai, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, Docker, AWS, LangChain, LangGraph, RAG, Openai, Anthropic, Claude, Ollama, Transformers, React, Next.js, Javascript, Node.Js, GIT, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>Hari Shanker Sharma qualifies as an eligible candidate with a total score of 73.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, PostgreSQL, Redis, Docker. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Low or dormant public GitHub activity. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Kiran Naregal scored 70.5/100 (AI 35.0/40, Python 20.0/30, Cloud 14.0/15, GitHub 0.0/10), led by observability and concurrency handling and stateful multi-agent orchestration (langgraph/crewai/autogen) Backed by embeddings-based retrieval system. Stack centers on Python, FastAPI, Docker, AWS. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -1559,22 +1559,22 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Jyandeep Baishya</t>
+          <t>Vivek Chimnani</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>craftzyan@gmail.com</t>
+          <t>vivekchimnani4231@gmail.com</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>6002590335</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>candidate_07.pdf</t>
+          <t>candidate_44.pdf</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1583,41 +1583,43 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>73</v>
+        <v>68.5</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>7.1</v>
+        <v>3.5</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P12" s="3" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0</v>
@@ -1636,12 +1638,12 @@
       </c>
       <c r="W12" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Redis, LangChain, LangGraph, RAG, ChromaDB, Tool Calling, React, Next.js, Typescript, Node.Js</t>
+          <t>Python, FastAPI, PostgreSQL, Redis, Docker, AWS, LangGraph, Claude, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd, Linux, Mongodb</t>
         </is>
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>Jyandeep Baishya qualifies as an eligible candidate with a total score of 73.0/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, Redis, LangChain, LangGraph. GitHub enrichment indicates: Veteran Builder (3.4 yrs on GitHub, 45 repos, 0 recent commits). 7 relevant Python/AI repositories identified. Primary area for review: No explicit testing (pytest/unit tests) mentioned. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 68.5/100, Vivek Chimnani stands out through automated testing / ci/cd pipeline, complemented by observability and concurrency handling. Plus stateful multi-agent orchestration (langgraph/crewai/autogen) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Redis, Docker maps to AI 24.0 and Python 27.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -1651,22 +1653,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Kiran Naregal</t>
+          <t>Yash Maini</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>kirnaregal7@gmail.com</t>
+          <t>mainiyash2@gmail.com</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>9964923041</t>
+          <t>+91-8920028757</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>candidate_47.pdf</t>
+          <t>candidate_13.pdf</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1675,25 +1677,25 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>70.5</v>
+        <v>68</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>8.76</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -1728,12 +1730,12 @@
       </c>
       <c r="W13" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Docker, AWS, LangChain, LangGraph, RAG, Openai, Anthropic, Claude, Ollama, Transformers, React, Next.js, Javascript, Node.Js, GIT, SQL, Mongodb</t>
+          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, GCP, AWS, LangChain, LangGraph, RAG, Faiss, Pinecone, Embeddings, Tool Calling, Openai, Claude, Pytorch, Tensorflow, Rest Api, Ci/Cd, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>Kiran Naregal qualifies as an eligible candidate with a total score of 70.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, Docker, AWS, LangChain. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Yash Maini scored 68.0/100 (AI 33.0/40, Python 22.0/30, Cloud 11.0/15, GitHub 0.0/10), led by automated testing / ci/cd pipeline and stateful multi-agent orchestration (langgraph/crewai/autogen) Backed by vector database retrieval (chromadb/faiss/pinecone/qdrant). Stack centers on Python, FastAPI, Flask, PostgreSQL. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -1743,22 +1745,22 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Krishan Kant</t>
+          <t>Prajwal A S</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>krishankantptu@gmail.com</t>
+          <t>prajwalas8999@gmail.com</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>+91-6204142591</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>candidate_09.pdf</t>
+          <t>candidate_22.pdf</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1767,25 +1769,27 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>69.5</v>
+        <v>68</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>25</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>7.33</v>
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1794,20 +1798,20 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P14" s="3" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="T14" s="3" t="n">
         <v>0</v>
@@ -1820,12 +1824,12 @@
       </c>
       <c r="W14" s="3" t="inlineStr">
         <is>
-          <t>Python, PostgreSQL, Redis, Docker, LangChain, RAG, Vector Search, Openai, React, Typescript, Javascript, Kafka, GIT, SQL, Mongodb, Java, Spring Boot</t>
+          <t>Python, FastAPI, Flask, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Ollama, React, Javascript, Rest Api, GIT, Linux, SQL</t>
         </is>
       </c>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>Krishan Kant qualifies as an eligible candidate with a total score of 69.5/100. The candidate demonstrates practical engineering capability highlighted by agentic workflow with tool/function calling, embeddings-based retrieval system, supported by core stack competencies in Python, PostgreSQL, Redis, Docker, LangChain. GitHub enrichment indicates: Veteran Builder (4.0 yrs on GitHub, 21 repos, 0 recent commits). 2 relevant Python/AI repositories identified. Primary area for review: No explicit testing (pytest/unit tests) mentioned. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 68.0/100, Prajwal A S stands out through embeddings-based retrieval system, complemented by async fastapi backend architecture. Plus postgresql with orm / schema migrations rounds out the build. Core evidence in Python, FastAPI, Flask, PostgreSQL, LangChain maps to AI 31.0 and Python 25.0 bands. GitHub profile: Active Builder (2.9 yrs on GitHub, 32 repos [29 original], 44 contributions in past year [0 commits]). 13 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -1835,22 +1839,22 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Vivek Chimnani</t>
+          <t>Jyandeep Baishya</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>vivekchimnani4231@gmail.com</t>
+          <t>craftzyan@gmail.com</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>6002590335</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>candidate_44.pdf</t>
+          <t>candidate_07.pdf</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1859,31 +1863,29 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>68.5</v>
+        <v>63</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>7.1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -1914,12 +1916,12 @@
       </c>
       <c r="W15" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Redis, Docker, AWS, LangGraph, Claude, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd, Linux, Mongodb</t>
+          <t>Python, FastAPI, Redis, LangChain, LangGraph, RAG, ChromaDB, Tool Calling, React, Next.js, Typescript, Node.Js</t>
         </is>
       </c>
       <c r="X15" s="3" t="inlineStr">
         <is>
-          <t>Vivek Chimnani qualifies as an eligible candidate with a total score of 68.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), async fastapi backend architecture, supported by core stack competencies in Python, FastAPI, PostgreSQL, Redis, Docker. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Low or dormant public GitHub activity. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 63.0/100, Jyandeep Baishya stands out through cloud infrastructure (aws/azure), complemented by full stack capability (react/next.js/typescript). Plus stateful multi-agent orchestration (langgraph/crewai/autogen) rounds out the build. Core evidence in Python, FastAPI, Redis, LangChain, LangGraph maps to AI 33.0 and Python 22.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -1929,22 +1931,22 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Prajwal A S</t>
+          <t>M Sai Kushith</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>prajwalas8999@gmail.com</t>
+          <t>msaikushith718@gmail.com</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91-7842732706</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>candidate_22.pdf</t>
+          <t>candidate_06.pdf</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1953,19 +1955,19 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="H16" s="3" t="n">
         <v>31</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>4</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L16" s="3" t="n">
         <v>0</v>
@@ -1977,25 +1979,25 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P16" s="3" t="n">
-        <v>2.9</v>
+        <v>1.3</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" s="3" t="n">
         <v>0</v>
@@ -2008,12 +2010,12 @@
       </c>
       <c r="W16" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Ollama, React, Javascript, Rest Api, GIT, Linux, SQL</t>
+          <t>Python, FastAPI, Django, PostgreSQL, LangChain, LangGraph, RAG, React, Typescript, GIT, Linux, SQL, Java</t>
         </is>
       </c>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>Prajwal A S qualifies as an eligible candidate with a total score of 65.0/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, Flask, PostgreSQL, LangChain. GitHub enrichment indicates: Active Developer (2.9 yrs on GitHub, 32 repos, 0 recent commits). 13 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 61.0/100, M Sai Kushith stands out through full stack capability (react/next.js/typescript), complemented by stateful multi-agent orchestration (langgraph/crewai/autogen). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, LangChain maps to AI 31.0 and Python 20.0 bands. GitHub profile: Active Builder (1.3 yrs on GitHub, 4 repos [4 original], 1 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -2023,22 +2025,22 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Priyanshu Kumar</t>
+          <t>Krishan Kant</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>krpriyanshu2805@gmail.com</t>
+          <t>krishankantptu@gmail.com</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>+91 8210008947</t>
+          <t>+91-6204142591</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>candidate_16.pdf</t>
+          <t>candidate_09.pdf</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2047,25 +2049,25 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>60.5</v>
+        <v>61</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>8</v>
+        <v>7.33</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -2074,14 +2076,14 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P17" s="3" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>0</v>
@@ -2100,12 +2102,12 @@
       </c>
       <c r="W17" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG, Pinecone, Embeddings, Tool Calling, React, Javascript, Node.Js, Kafka, GIT, Mongodb</t>
+          <t>Python, PostgreSQL, Redis, Docker, LangChain, RAG, Vector Search, Openai, React, Typescript, Javascript, Kafka, GIT, SQL, Mongodb, Java, Spring Boot</t>
         </is>
       </c>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t>Priyanshu Kumar qualifies as an eligible candidate with a total score of 60.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, PostgreSQL, LangChain, LangGraph. GitHub enrichment indicates: Active Developer (3.3 yrs on GitHub, 13 repos, 0 recent commits). 7 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 61.0/100, Krishan Kant stands out through distributed task queues (celery/rabbitmq/kafka), complemented by observability and concurrency handling. Plus agentic workflow with tool/function calling rounds out the build. Core evidence in Python, PostgreSQL, Redis, Docker, LangChain maps to AI 23.0 and Python 25.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2199,7 @@
       </c>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>Nevil Jasmin Mehta qualifies as an eligible candidate with a total score of 60.5/100. The candidate demonstrates practical engineering capability highlighted by vector database retrieval (chromadb/faiss/pinecone/qdrant), async fastapi backend architecture, supported by core stack competencies in Python, FastAPI, Django, Flask, PostgreSQL. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Low or dormant public GitHub activity. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Nevil Jasmin Mehta (60.5/100) impressed with vector database retrieval (chromadb/faiss/pinecone/qdrant) alongside async fastapi backend architecture. Also notable: postgresql with orm / schema migrations. Depth spans Python, FastAPI, Django, Flask, PostgreSQL, Redis (cloud 14.0/15, GitHub 0.0/10). Activity: GitHub API rate limit exceeded; skipped enrichment. Interview focus should be low or dormant public github activity, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -2207,22 +2209,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>P V Jayavardhana Sai</t>
+          <t>Thejeshwaar Paasila</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>pvjayavardhan6@gmail.com</t>
+          <t>thejeshwaarp@gmail.com</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 6303204136</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>candidate_19.pdf</t>
+          <t>candidate_26.pdf</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2234,44 +2236,46 @@
         <v>59.5</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>8.6</v>
+        <v>2</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Emerging Developer</t>
         </is>
       </c>
       <c r="P19" s="3" t="n">
-        <v>3.7</v>
+        <v>2.3</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S19" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T19" s="3" t="n">
         <v>0</v>
@@ -2284,12 +2288,12 @@
       </c>
       <c r="W19" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, Docker, AWS, RAG, Ollama, Transformers, Pytorch, Tensorflow, React, Javascript, GIT, SQL, Java</t>
+          <t>Python, Flask, PostgreSQL, Docker, Google Cloud, RAG, Openai, Gemini, Claude, Transformers, React, Next.js, Typescript, Javascript, Node.Js, GIT, Ci/Cd, Linux, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X19" s="3" t="inlineStr">
         <is>
-          <t>P V Jayavardhana Sai qualifies as an eligible candidate with a total score of 59.5/100. The candidate demonstrates practical engineering capability highlighted by basic agent implementation, embeddings-based retrieval system, supported by core stack competencies in Python, Flask, Docker, AWS, RAG. GitHub enrichment indicates: Active Developer (3.7 yrs on GitHub, 8 repos, 0 recent commits). 5 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 59.5/100, Thejeshwaar Paasila stands out through modern python backend framework (fastapi/django), complemented by postgresql with orm / schema migrations. Plus docker containerization &amp; deployment rounds out the build. Core evidence in Python, Flask, PostgreSQL, Docker, Google Cloud maps to AI 16.0 and Python 20.0 bands. GitHub profile: Emerging Developer (2.3 yrs on GitHub, 3 repos [2 original], 10 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -2299,22 +2303,22 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>M Sai Kushith</t>
+          <t>Vivek Shekhawat</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>msaikushith718@gmail.com</t>
+          <t>vivekshekhawatofficial1592002@gmail.com</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>+91-7842732706</t>
+          <t>+91-7734911626</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>candidate_06.pdf</t>
+          <t>candidate_39.pdf</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2323,13 +2327,13 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>58.5</v>
+        <v>59</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>4</v>
@@ -2338,34 +2342,32 @@
         <v>3.5</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>9.140000000000001</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P20" s="3" t="n">
-        <v>1.3</v>
+        <v>4.1</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="R20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" s="3" t="n">
         <v>0</v>
@@ -2378,12 +2380,12 @@
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, PostgreSQL, LangChain, LangGraph, RAG, React, Typescript, GIT, Linux, SQL, Java</t>
+          <t>Python, Django, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Vector Search, Ollama, React, Next.js, Javascript, Node.Js, GIT, SQL, Java</t>
         </is>
       </c>
       <c r="X20" s="3" t="inlineStr">
         <is>
-          <t>M Sai Kushith qualifies as an eligible candidate with a total score of 58.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, Django, PostgreSQL, LangChain. GitHub enrichment indicates: Active Developer (1.3 yrs on GitHub, 4 repos, 0 recent commits). 1 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Vivek Shekhawat scored 59.0/100 (AI 27.0/40, Python 23.0/30, Cloud 4.0/15, GitHub 3.5/10), led by postgresql with orm / schema migrations and full stack capability (react/next.js/typescript) Backed by observability and concurrency handling. Stack centers on Python, Django, PostgreSQL, LangChain. GitHub: Veteran Builder (4.1 yrs on GitHub, 15 repos [0 original], 1 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Watch-item: no explicit testing (pytest/unit tests) mentioned. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -2393,22 +2395,22 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Thejeshwaar Paasila</t>
+          <t>Pavani A</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>thejeshwaarp@gmail.com</t>
+          <t>pavani10112004@gmail.com</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>+91 6303204136</t>
+          <t>+919742542200</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>candidate_26.pdf</t>
+          <t>candidate_38.pdf</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2417,49 +2419,47 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>56.5</v>
+        <v>58</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>20</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M21" s="2" t="n">
+        <v>9.710000000000001</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Emerging Developer</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P21" s="3" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="R21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="3" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="T21" s="3" t="n">
         <v>0</v>
@@ -2472,12 +2472,12 @@
       </c>
       <c r="W21" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, PostgreSQL, Docker, Google Cloud, RAG, Openai, Gemini, Claude, Transformers, React, Next.js, Typescript, Javascript, Node.Js, GIT, Ci/Cd, Linux, SQL, Mongodb</t>
+          <t>Python, FastAPI, Django, Flask, PostgreSQL, Docker, Tensorflow, React, Next.js, Javascript, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X21" s="3" t="inlineStr">
         <is>
-          <t>Thejeshwaar Paasila qualifies as an eligible candidate with a total score of 56.5/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, modern python backend framework (fastapi/django), supported by core stack competencies in Python, Flask, PostgreSQL, Docker, Google Cloud. GitHub enrichment indicates: Emerging Developer (2.3 yrs on GitHub, 3 repos, 0 recent commits). 1 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 58.0/100, Pavani A stands out through postgresql with orm / schema migrations, complemented by docker containerization &amp; deployment. Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, Django, Flask, PostgreSQL maps to AI 20.0 and Python 20.0 bands. GitHub profile: Active Builder (1.9 yrs on GitHub, 16 repos [0 original], 19 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -2487,22 +2487,22 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Shubhanshu Navadiya</t>
+          <t>Aditi Kala</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>subhnavadiya@gmail.com</t>
+          <t>aditi25.kala@gmail.com</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>+91 9031132507</t>
+          <t>+91-8368407039</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>candidate_12.pdf</t>
+          <t>candidate_37.pdf</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2511,25 +2511,27 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>8.1</v>
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -2538,38 +2540,38 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P22" s="3" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="R22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>0</v>
+        <v>567</v>
       </c>
       <c r="T22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="V22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W22" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant, Weaviate, Embeddings, Openai, Gemini, Ollama, Transformers, Pytorch, GIT, SQL</t>
+          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, Google Cloud, Gemini, Pytorch, Tensorflow, React, Node.Js, GIT, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X22" s="3" t="inlineStr">
         <is>
-          <t>Shubhanshu Navadiya qualifies as an eligible candidate with a total score of 56.0/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), vector database retrieval (chromadb/faiss/pinecone/qdrant), supported by core stack competencies in Python, FastAPI, LangChain, LlamaIndex, RAG. GitHub enrichment indicates: Active Developer (4.0 yrs on GitHub, 25 repos, 0 recent commits). 14 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Aditi Kala scored 58.0/100 (AI 14.0/40, Python 23.0/30, Cloud 15.0/15, GitHub 6.0/10), led by basic agent implementation and embeddings-based retrieval system Backed by modern python backend framework (fastapi/django). Stack centers on Python, FastAPI, Flask, PostgreSQL. GitHub: Veteran Builder (3.5 yrs on GitHub, 53 repos [0 original], 567 contributions in past year [0 commits, 27 PRs]). 0 relevant Python/AI repositories identified. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -2579,22 +2581,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Vivek Shekhawat</t>
+          <t>Priyanshu Kumar</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>vivekshekhawatofficial1592002@gmail.com</t>
+          <t>krpriyanshu2805@gmail.com</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>+91-7734911626</t>
+          <t>+91 8210008947</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>candidate_39.pdf</t>
+          <t>candidate_16.pdf</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2606,10 +2608,10 @@
         <v>55.5</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>4</v>
@@ -2621,7 +2623,7 @@
         <v>1.5</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>9.140000000000001</v>
+        <v>8</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
@@ -2656,12 +2658,12 @@
       </c>
       <c r="W23" s="3" t="inlineStr">
         <is>
-          <t>Python, Django, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Vector Search, Ollama, React, Next.js, Javascript, Node.Js, GIT, SQL, Java</t>
+          <t>Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG, Pinecone, Embeddings, Tool Calling, React, Javascript, Node.Js, Kafka, GIT, Mongodb</t>
         </is>
       </c>
       <c r="X23" s="3" t="inlineStr">
         <is>
-          <t>Vivek Shekhawat qualifies as an eligible candidate with a total score of 55.5/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), embeddings-based retrieval system, supported by core stack competencies in Python, Django, PostgreSQL, LangChain, LangGraph. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Priyanshu Kumar scored 55.5/100 (AI 28.0/40, Python 22.0/30, Cloud 4.0/15, GitHub 0.0/10), led by stateful multi-agent orchestration (langgraph/crewai/autogen) and vector database retrieval (chromadb/faiss/pinecone/qdrant) Backed by async fastapi backend architecture. Stack centers on Python, FastAPI, PostgreSQL, LangChain. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -2671,22 +2673,22 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Raj Thumar</t>
+          <t>P V Jayavardhana Sai</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>thumarraj999@gmail.com</t>
+          <t>pvjayavardhan6@gmail.com</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>+91 9104382983</t>
+          <t>+91 99663 46173</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>candidate_40.pdf</t>
+          <t>candidate_19.pdf</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2698,10 +2700,10 @@
         <v>54.5</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>14</v>
@@ -2710,12 +2712,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>8.6</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, PostgreSQL, Redis, Docker, AWS, RAG, Openai, Gemini, React, Typescript, Javascript, Node.Js, Graphql, Kafka, Mongodb</t>
+          <t>Python, Flask, Docker, AWS, RAG, Ollama, Transformers, Pytorch, Tensorflow, React, Javascript, GIT, SQL, Java</t>
         </is>
       </c>
       <c r="X24" s="3" t="inlineStr">
         <is>
-          <t>Raj Thumar qualifies as an eligible candidate with a total score of 54.5/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, modern python backend framework (fastapi/django), supported by core stack competencies in Python, Flask, PostgreSQL, Redis, Docker. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Low or dormant public GitHub activity. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 54.5/100, P V Jayavardhana Sai stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, Flask, Docker, AWS, RAG maps to AI 22.0 and Python 17.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -2765,22 +2765,22 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Harsha A</t>
+          <t>Raj Thumar</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>harshaarun2608@gmail.com</t>
+          <t>thumarraj999@gmail.com</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 9104382983</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>candidate_15.pdf</t>
+          <t>candidate_40.pdf</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -2789,13 +2789,13 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>54</v>
+        <v>54.5</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J25" s="3" t="n">
         <v>14</v>
@@ -2804,19 +2804,21 @@
         <v>0</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>7.55</v>
+        <v>3.5</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Unlinked / Missing</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P25" s="3" t="n">
@@ -2842,12 +2844,12 @@
       </c>
       <c r="W25" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Docker, Azure, Tensorflow, React, Javascript, Node.Js, SQL, Java</t>
+          <t>Python, Flask, PostgreSQL, Redis, Docker, AWS, RAG, Openai, Gemini, React, Typescript, Javascript, Node.Js, Graphql, Kafka, Mongodb</t>
         </is>
       </c>
       <c r="X25" s="3" t="inlineStr">
         <is>
-          <t>Harsha A qualifies as an eligible candidate with a total score of 54.0/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, ai evaluation pipeline (ragas/langsmith/trulens), supported by core stack competencies in Python, FastAPI, PostgreSQL, Docker, Azure. GitHub enrichment indicates: No public GitHub profile provided. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 54.5/100, Raj Thumar stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, Flask, PostgreSQL, Redis, Docker maps to AI 12.0 and Python 25.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -2857,22 +2859,22 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Aditi Kala</t>
+          <t>Harsha A</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>aditi25.kala@gmail.com</t>
+          <t>harshaarun2608@gmail.com</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>+91-8368407039</t>
+          <t>+91-9113869665</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>candidate_37.pdf</t>
+          <t>candidate_15.pdf</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -2881,36 +2883,34 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H26" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J26" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="I26" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="J26" s="3" t="n">
-        <v>15</v>
-      </c>
       <c r="K26" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M26" s="2" t="n">
+        <v>7.55</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Unlinked / Missing</t>
         </is>
       </c>
       <c r="P26" s="3" t="n">
@@ -2936,12 +2936,12 @@
       </c>
       <c r="W26" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, Google Cloud, Gemini, Pytorch, Tensorflow, React, Node.Js, GIT, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, PostgreSQL, Docker, Azure, Tensorflow, React, Javascript, Node.Js, SQL, Java</t>
         </is>
       </c>
       <c r="X26" s="3" t="inlineStr">
         <is>
-          <t>Aditi Kala qualifies as an eligible candidate with a total score of 52.0/100. The candidate demonstrates practical engineering capability highlighted by basic agent implementation, embeddings-based retrieval system, supported by core stack competencies in Python, FastAPI, Flask, PostgreSQL, Postgres. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 54.0/100, Harsha A stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Docker, Azure maps to AI 20.0 and Python 20.0 bands. GitHub profile: No public GitHub profile provided. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -2951,22 +2951,22 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Pavani A</t>
+          <t>Shubhanshu Navadiya</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>pavani10112004@gmail.com</t>
+          <t>subhnavadiya@gmail.com</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 9031132507</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>candidate_38.pdf</t>
+          <t>candidate_12.pdf</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2975,16 +2975,16 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>0</v>
@@ -2993,7 +2993,7 @@
         <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>9.710000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
@@ -3028,12 +3028,12 @@
       </c>
       <c r="W27" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, Flask, PostgreSQL, Docker, Tensorflow, React, Next.js, Javascript, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant, Weaviate, Embeddings, Openai, Gemini, Ollama, Transformers, Pytorch, GIT, SQL</t>
         </is>
       </c>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t>Pavani A qualifies as an eligible candidate with a total score of 52.0/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, ai evaluation pipeline (ragas/langsmith/trulens), supported by core stack competencies in Python, FastAPI, Django, Flask, PostgreSQL. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Shubhanshu Navadiya (51.0/100) impressed with stateful multi-agent orchestration (langgraph/crewai/autogen) alongside vector database retrieval (chromadb/faiss/pinecone/qdrant). Also notable: ai evaluation pipeline (ragas/langsmith/trulens). Depth spans Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant (cloud 0.0/15, GitHub 0.0/10). Activity: GitHub API rate limit exceeded; skipped enrichment. Interview focus should be low or dormant public github activity, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="X28" s="3" t="inlineStr">
         <is>
-          <t>Aswin Raj R qualifies as an eligible candidate with a total score of 48.0/100. The candidate demonstrates practical engineering capability highlighted by agentic workflow with tool/function calling, embeddings-based retrieval system, supported by core stack competencies in Python, AWS, LangChain, RAG, Openai. GitHub enrichment indicates: GitHub API rate limit exceeded; skipped enrichment. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Aswin Raj R scored 48.0/100 (AI 23.0/40, Python 17.0/30, Cloud 8.0/15, GitHub 0.0/10), led by embeddings-based retrieval system and cloud infrastructure (aws/azure) Backed by full stack capability (react/next.js/typescript). Stack centers on Python, AWS, LangChain, RAG. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -3137,22 +3137,22 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Higher Secondary Science Pcmb</t>
+          <t>Annisha S</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>manojkumar.k.r0904@gmail.com</t>
+          <t>annishasaravanan83@gmail.com</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9361112081</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>candidate_21.pdf</t>
+          <t>candidate_23.pdf</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3161,25 +3161,25 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>44.5</v>
+        <v>43</v>
       </c>
       <c r="H29" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I29" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="I29" s="3" t="n">
-        <v>17</v>
-      </c>
       <c r="J29" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="L29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>7.65</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
@@ -3188,14 +3188,14 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Emerging Developer</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P29" s="3" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R29" s="3" t="n">
         <v>0</v>
@@ -3214,12 +3214,12 @@
       </c>
       <c r="W29" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, Pytorch, Tensorflow, React, GIT, SQL, Java</t>
+          <t>Python, FastAPI, PostgreSQL, Azure, LangGraph, Openai, React, GIT, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X29" s="3" t="inlineStr">
         <is>
-          <t>Higher Secondary Science Pcmb qualifies as an eligible candidate with a total score of 44.5/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, ai evaluation pipeline (ragas/langsmith/trulens), supported by core stack competencies in Python, Flask, Pytorch, Tensorflow, React. GitHub enrichment indicates: Emerging Developer (1.9 yrs on GitHub, 1 repos, 0 recent commits). 1 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 43.0/100, Annisha S stands out through postgresql with orm / schema migrations, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Azure, LangGraph maps to AI 15.0 and Python 20.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -3229,22 +3229,22 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Annisha S</t>
+          <t>Atul Kumar</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>annishasaravanan83@gmail.com</t>
+          <t>atulofficial02@gmail.com</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>9361112081</t>
+          <t>+91-9368449979</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>candidate_23.pdf</t>
+          <t>candidate_25.pdf</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3253,25 +3253,27 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J30" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K30" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K30" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="L30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M30" s="2" t="n">
-        <v>8.720000000000001</v>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
@@ -3280,20 +3282,20 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P30" s="3" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="S30" s="3" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="T30" s="3" t="n">
         <v>0</v>
@@ -3306,12 +3308,12 @@
       </c>
       <c r="W30" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Azure, LangGraph, Openai, React, GIT, SQL, Mongodb</t>
+          <t>Python, Flask, GCP, Google Cloud, Gemini, Rest Api, GIT, SQL</t>
         </is>
       </c>
       <c r="X30" s="3" t="inlineStr">
         <is>
-          <t>Annisha S qualifies as an eligible candidate with a total score of 44.0/100. The candidate demonstrates practical engineering capability highlighted by stateful multi-agent orchestration (langgraph/crewai/autogen), modern python backend framework (fastapi/django), supported by core stack competencies in Python, FastAPI, PostgreSQL, Azure, LangGraph. GitHub enrichment indicates: Active Developer (2.3 yrs on GitHub, 4 repos, 0 recent commits). 0 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Atul Kumar (42.0/100) impressed with embeddings-based retrieval system alongside modern python backend framework (fastapi/django). Also notable: gcp cloud deployment experience. Depth spans Python, Flask, GCP, Google Cloud, Gemini, Rest Api (cloud 5.0/15, GitHub 8.0/10). Activity: Active Builder (1.7 yrs on GitHub, 9 repos [9 original], 42 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -3321,22 +3323,22 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Dornipadu Karthika Chaitrika</t>
+          <t>Higher Secondary Science Pcmb</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>dornipadukarthi@gmail.com</t>
+          <t>manojkumar.k.r0904@gmail.com</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>+91-9014209602</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>candidate_24.pdf</t>
+          <t>candidate_21.pdf</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -3345,25 +3347,25 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>8.43</v>
+        <v>7.65</v>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
@@ -3372,14 +3374,14 @@
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P31" s="3" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="R31" s="3" t="n">
         <v>0</v>
@@ -3398,12 +3400,12 @@
       </c>
       <c r="W31" s="3" t="inlineStr">
         <is>
-          <t>Python, Django, Flask, RAG, Embeddings, Gemini, Javascript</t>
+          <t>Python, Flask, Pytorch, Tensorflow, React, GIT, SQL, Java</t>
         </is>
       </c>
       <c r="X31" s="3" t="inlineStr">
         <is>
-          <t>Dornipadu Karthika Chaitrika qualifies as an eligible candidate with a total score of 40.0/100. The candidate demonstrates practical engineering capability highlighted by basic agent implementation, embeddings-based retrieval system, supported by core stack competencies in Python, Django, Flask, RAG, Embeddings. GitHub enrichment indicates: Active Developer (2.6 yrs on GitHub, 20 repos, 0 recent commits). 12 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 41.0/100, Higher Secondary Science Pcmb stands out through modern python backend framework (fastapi/django), complemented by full stack capability (react/next.js/typescript). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, Flask, Pytorch, Tensorflow, React maps to AI 20.0 and Python 17.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -3413,22 +3415,22 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Atul Kumar</t>
+          <t>Dornipadu Karthika Chaitrika</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>atulofficial02@gmail.com</t>
+          <t>dornipadukarthi@gmail.com</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>+91-9368449979</t>
+          <t>+91-9014209602</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>candidate_25.pdf</t>
+          <t>candidate_24.pdf</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -3437,27 +3439,25 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H32" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="I32" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="I32" s="3" t="n">
-        <v>17</v>
-      </c>
       <c r="J32" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M32" s="2" t="n">
+        <v>8.43</v>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
@@ -3466,14 +3466,14 @@
       </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P32" s="3" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="R32" s="3" t="n">
         <v>0</v>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="W32" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, GCP, Google Cloud, Gemini, Rest Api, GIT, SQL</t>
+          <t>Python, Django, Flask, RAG, Embeddings, Gemini, Javascript</t>
         </is>
       </c>
       <c r="X32" s="3" t="inlineStr">
         <is>
-          <t>Atul Kumar qualifies as an eligible candidate with a total score of 39.0/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, modern python backend framework (fastapi/django), supported by core stack competencies in Python, Flask, GCP, Google Cloud, Gemini. GitHub enrichment indicates: Active Developer (1.7 yrs on GitHub, 9 repos, 0 recent commits). 7 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>Dornipadu Karthika Chaitrika scored 35.0/100 (AI 23.0/40, Python 12.0/30, Cloud 0.0/15, GitHub 0.0/10), led by basic agent implementation and embeddings-based retrieval system Backed by modern python backend framework (fastapi/django). Stack centers on Python, Django, Flask, RAG. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>30.5</v>
+        <v>28</v>
       </c>
       <c r="H33" s="3" t="n">
         <v>7</v>
@@ -3543,7 +3543,7 @@
         <v>4</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="L33" s="3" t="n">
         <v>0</v>
@@ -3558,14 +3558,14 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Active Developer</t>
+          <t>Unverified (Rate Limited)</t>
         </is>
       </c>
       <c r="P33" s="3" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="R33" s="3" t="n">
         <v>0</v>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="X33" s="3" t="inlineStr">
         <is>
-          <t>Saif Ali Nagori qualifies as an eligible candidate with a total score of 30.5/100. The candidate demonstrates practical engineering capability highlighted by embeddings-based retrieval system, modern python backend framework (fastapi/django), supported by core stack competencies in Python, FastAPI, Flask, RAG, React. GitHub enrichment indicates: Active Developer (3.1 yrs on GitHub, 26 repos, 0 recent commits). 0 relevant Python/AI repositories identified. Primary area for review: Limited Redis or backend caching evidence. Overall, this profile exhibits solid engineering depth and the requisite hands-on exposure to modern agentic systems to succeed in the SDE AI internship.</t>
+          <t>At 28.0/100, Saif Ali Nagori stands out through modern python backend framework (fastapi/django), complemented by full stack capability (react/next.js/typescript). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, FastAPI, Flask, RAG, React maps to AI 7.0 and Python 17.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 89558-87066</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="X34" s="3" t="inlineStr">
         <is>
-          <t>Aabhar Gupta was marked ineligible during screening due to no evidence of python stack, no ai/agentic project evidence. While the candidate presents background in PostgreSQL, Redis, Google Cloud, React, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Aabhar Gupta does not advance (ineligible, 0.0/100). Core gap: no evidence of python stack, no ai/agentic project evidence. While PostgreSQL, Redis, Google Cloud, React, Javascript shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="X35" s="3" t="inlineStr">
         <is>
-          <t>Agam Jain was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, FastAPI, PostgreSQL, Redis, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Agam Jain ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, FastAPI, PostgreSQL, Redis, Docker) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="X36" s="3" t="inlineStr">
         <is>
-          <t>Anjali Patil was marked ineligible during screening due to no evidence of python stack, no ai/agentic project evidence. While the candidate presents background in PostgreSQL, Redis, Docker, Javascript, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Anjali Patil was marked ineligible at 0.0/100 due to no evidence of python stack, no ai/agentic project evidence. Background shows PostgreSQL, Redis, Docker, Javascript, GIT, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="X37" s="3" t="inlineStr">
         <is>
-          <t>Gayathri Palraj was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, React, Typescript, Javascript, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Gayathri Palraj was marked ineligible at 0.0/100 due to no ai/agentic project evidence. Background shows Python, React, Typescript, Javascript, Node.Js, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="X38" s="3" t="inlineStr">
         <is>
-          <t>Harshit Kumar Mishra was marked ineligible during screening due to no evidence of python stack, no ai/agentic project evidence. While the candidate presents background in PostgreSQL, Redis, Docker, GCP, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Harshit Kumar Mishra was marked ineligible at 0.0/100 due to no evidence of python stack, no ai/agentic project evidence. Background shows PostgreSQL, Redis, Docker, GCP, AWS, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="X39" s="3" t="inlineStr">
         <is>
-          <t>Jaya Nandi was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, AWS, React, Javascript, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Jaya Nandi was marked ineligible at 0.0/100 due to no ai/agentic project evidence. Background shows Python, AWS, React, Javascript, Rest Api, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="X40" s="3" t="inlineStr">
         <is>
-          <t>Kartikay Sinha was marked ineligible during screening due to no evidence of python stack, no ai/agentic project evidence. While the candidate presents background in Docker, React, Next.js, Typescript, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Kartikay Sinha ineligible (0.0/100) — no evidence of python stack, no ai/agentic project evidence. Seen skills (Docker, React, Next.js, Typescript, Javascript) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="X41" s="3" t="inlineStr">
         <is>
-          <t>Md Azizul Islam was marked ineligible during screening due to no evidence of python stack. While the candidate presents background in PostgreSQL, Redis, AWS, RAG, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Md Azizul Islam ineligible (0.0/100) — no evidence of python stack. Seen skills (PostgreSQL, Redis, AWS, RAG, Embeddings) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4445,7 @@
       </c>
       <c r="X42" s="3" t="inlineStr">
         <is>
-          <t>Mukul Pal was marked ineligible during screening due to no evidence of python stack. While the candidate presents background in PostgreSQL, Redis, Docker, AWS, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Mukul Pal ineligible (0.0/100) — no evidence of python stack. Seen skills (PostgreSQL, Redis, Docker, AWS, Openai) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4539,7 +4539,7 @@
       </c>
       <c r="X43" s="3" t="inlineStr">
         <is>
-          <t>Nidhi Km was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, AWS, Tensorflow, React, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Nidhi Km ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, AWS, Tensorflow, React, Javascript) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="X44" s="3" t="inlineStr">
         <is>
-          <t>Nisarga H S was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, Claude, Node.Js, GIT, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Nisarga H S was marked ineligible at 0.0/100 due to no ai/agentic project evidence. Background shows Python, Claude, Node.Js, GIT, Ci/Cd, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
         </is>
       </c>
     </row>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="X45" s="3" t="inlineStr">
         <is>
-          <t>Parshuram Kumar was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, Django, Flask, Redis, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Parshuram Kumar ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Django, Flask, Redis, Docker) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="X46" s="3" t="inlineStr">
         <is>
-          <t>Programming Language Python was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, React, Javascript, GIT, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Programming Language Python does not advance (ineligible, 0.0/100). Core gap: no ai/agentic project evidence. While Python, React, Javascript, GIT, SQL shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 73228 09264</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="X47" s="3" t="inlineStr">
         <is>
-          <t>Shivam Raj was marked ineligible during screening due to no evidence of python stack, no ai/agentic project evidence. While the candidate presents background in Docker, Azure, React, Next.js, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Shivam Raj does not advance (ineligible, 0.0/100). Core gap: no evidence of python stack, no ai/agentic project evidence. While Docker, Azure, React, Next.js, Typescript shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="X48" s="3" t="inlineStr">
         <is>
-          <t>Shreya Chauhan was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, Redis, React, Javascript, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Shreya Chauhan does not advance (ineligible, 0.0/100). Core gap: no ai/agentic project evidence. While Python, Redis, React, Javascript, Node.Js shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 9353172296</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="X49" s="3" t="inlineStr">
         <is>
-          <t>Vikram Madhyasta was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, Docker, Kubernetes, AWS, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Vikram Madhyasta was marked ineligible at 0.0/100 due to no ai/agentic project evidence. Background shows Python, Docker, Kubernetes, AWS, Openai, but the resume lacks concrete Python backend work and verifiable agentic, RAG, or LLM-tooling evidence. For this SDE AI internship the bar is shipped Python services plus agent orchestration, tool calling, or vector retrieval. This profile does not clear that baseline, though relevant Python building would change the outcome.</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="X50" s="3" t="inlineStr">
         <is>
-          <t>Vishwas Badiger was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, Flask, React, Javascript, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Vishwas Badiger ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Flask, React, Javascript, Node.Js) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="X51" s="3" t="inlineStr">
         <is>
-          <t>Yuvaraj R was marked ineligible during screening due to no ai/agentic project evidence. While the candidate presents background in Python, Django, PostgreSQL, Docker, the profile lacks practical evidence of Python backend development and demonstrable exposure to agentic, RAG, or LLM-based workflows. For this SDE internship, candidates must demonstrate functional experience building with Python services alongside agent orchestration, tool calling, or vector retrieval pipelines. Consequently, this profile does not meet the mandatory baseline criteria for further scoring consideration.</t>
+          <t>Screening result: Yuvaraj R ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Django, PostgreSQL, Docker, Rest Api) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update README with video demo link, UI showcase screenshots, and documentation
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -489,7 +489,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
@@ -815,22 +815,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Gourab Das</t>
+          <t>Sumaiya Sultana Shaik</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>gourabdas1307@gmail.com</t>
+          <t>sultanasumaiya623@gmail.com</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>+91-7002572852</t>
+          <t>+91 97015 28467</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>candidate_17.pdf</t>
+          <t>candidate_28.pdf</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>81.5</v>
+        <v>82.5</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>10</v>
@@ -856,10 +856,8 @@
       <c r="L4" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M4" s="2" t="n">
+        <v>7.1</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -868,38 +866,38 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
-        <v>6.3</v>
+        <v>2.7</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="S4" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="T4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, Flask, PostgreSQL, Redis, Docker, AWS, LangChain, LangGraph, RAG, React, Kafka, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java, Spring Boot</t>
+          <t>Python, FastAPI, PostgreSQL, Docker, GCP, LangChain, LangGraph, RAG, React, Typescript, Graphql, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Gourab Das (81.5/100) impressed with advanced rag with hybrid search and reranking alongside async fastapi backend architecture. Also notable: postgresql with orm / schema migrations. Depth spans Python, FastAPI, Django, Flask, PostgreSQL, Redis (cloud 14.0/15, GitHub 10.0/10). Activity: Veteran Builder (6.3 yrs on GitHub, 21 repos [12 original], 3 contributions in past year [0 commits]). 4 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
+          <t>At 82.5/100, Sumaiya Sultana Shaik stands out through stateful multi-agent orchestration (langgraph/crewai/autogen), complemented by embeddings-based retrieval system. Plus modern python backend framework (fastapi/django) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Docker, GCP maps to AI 31.0 and Python 23.0 bands. GitHub profile: Active Builder (2.7 yrs on GitHub, 29 repos [29 original], 13 contributions in past year [0 commits], 3 stars). 14 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -909,22 +907,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Vaibhav Wakde</t>
+          <t>Hari Shanker Sharma</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>vaibhavwakde266@gmail.com</t>
+          <t>harishankersharma648@gmail.com</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>+91-9307600143</t>
+          <t>+91 8801109700</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>candidate_33.pdf</t>
+          <t>candidate_41.pdf</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -933,19 +931,19 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>75.5</v>
+        <v>82.5</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>3.5</v>
@@ -966,16 +964,16 @@
         </is>
       </c>
       <c r="P5" s="3" t="n">
-        <v>3.5</v>
+        <v>6.3</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>12</v>
+        <v>116</v>
       </c>
       <c r="T5" s="3" t="n">
         <v>0</v>
@@ -984,16 +982,16 @@
         <v>0</v>
       </c>
       <c r="V5" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W5" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, Docker, AWS, LangChain, LangGraph, LlamaIndex, RAG, ChromaDB, Weaviate, Tool Calling, Openai, Ollama, Transformers, Javascript, Pytest, GIT, SQL</t>
+          <t>Python, FastAPI, PostgreSQL, Redis, Docker, Kubernetes, AWS, LangChain, LangGraph, RAG, Qdrant, Embeddings, Vector Search, Openai, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>Vaibhav Wakde (75.5/100) impressed with cloud infrastructure (aws/azure) alongside strong public github footprint (veteran builder). Also notable: automated testing / ci/cd pipeline. Depth spans Python, FastAPI, Flask, Docker, AWS, LangChain (cloud 10.0/15, GitHub 10.0/10). Activity: Veteran Builder (3.5 yrs on GitHub, 10 repos [10 original], 12 contributions in past year [0 commits]). 4 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
+          <t>Hari Shanker Sharma (82.5/100) impressed with redis caching / in-memory store alongside docker containerization &amp; deployment. Also notable: cloud infrastructure (aws/azure). Depth spans Python, FastAPI, PostgreSQL, Redis, Docker, Kubernetes (cloud 14.0/15, GitHub 9.0/10). Activity: Veteran Builder (6.3 yrs on GitHub, 30 repos [29 original], 116 contributions in past year [0 commits], 5 stars). 6 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1003,22 +1001,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Arunima Saha</t>
+          <t>Arjun Kumar</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>arunimasaha11@gmail.com</t>
+          <t>roy.prajapat.143@gmail.com</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>+91 9187656193</t>
+          <t>+91-6396303191</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>candidate_43.pdf</t>
+          <t>candidate_08.pdf</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1027,47 +1025,47 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>75.5</v>
+        <v>81.5</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Unlinked / Missing</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>0</v>
+        <v>226</v>
       </c>
       <c r="T6" s="3" t="n">
         <v>0</v>
@@ -1076,16 +1074,16 @@
         <v>0</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS, LangChain, LangGraph, RAG, Pinecone, Embeddings, Vector Search, Tool Calling, Openai, Gemini, Transformers, Rest Api, GIT, SQL</t>
+          <t>Python, FastAPI, Django, PostgreSQL, AWS, LangChain, LangGraph, RAG, Embeddings, Gemini, Tensorflow, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>Arunima Saha (75.5/100) impressed with advanced rag with hybrid search and reranking alongside ai evaluation pipeline (ragas/langsmith/trulens). Also notable: modern python backend framework (fastapi/django). Depth spans Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS (cloud 11.0/15, GitHub 0.0/10). Activity: No public GitHub profile provided. Interview focus should be no explicit testing (pytest/unit tests) mentioned, but overall internship readiness is high.</t>
+          <t>Arjun’s standout strength is designing stateful multi-agent systems with LangGraph, supported by a robust Python FastAPI backend. His portfolio highlights 13 relevant AI repositories, including an embeddings-based retrieval pipeline using LangChain and PostgreSQL. While his GitHub activity shows sustained building over three years, the absence of Redis or backend caching evidence remains a notable technical gap. Still, his focus on complex orchestration and RAG architectures makes him a strong fit for our high-volume AI infrastructure team.</t>
         </is>
       </c>
     </row>
@@ -1095,22 +1093,22 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Abhinav Mishra</t>
+          <t>Gourab Das</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>abhinavmishra3322@gmail.com</t>
+          <t>gourabdas1307@gmail.com</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>+91 7701956829</t>
+          <t>+91-7002572852</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>candidate_10.pdf</t>
+          <t>candidate_17.pdf</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1119,16 +1117,16 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>73.5</v>
+        <v>81.5</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>27</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>10</v>
@@ -1152,34 +1150,34 @@
         </is>
       </c>
       <c r="P7" s="3" t="n">
-        <v>3.4</v>
+        <v>6.3</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>4315</v>
+        <v>3</v>
       </c>
       <c r="T7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V7" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Redis, Azure, LangGraph, RAG, Openai, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd</t>
+          <t>Python, FastAPI, Django, Flask, PostgreSQL, Redis, Docker, AWS, LangChain, LangGraph, RAG, React, Kafka, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java, Spring Boot</t>
         </is>
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>Abhinav’s 3.4-year GitHub tenure reveals a veteran builder with 28 original repositories, proving sustained commitment beyond typical intern portfolios. His technical depth shines through stateful multi-agent orchestration using LangGraph and robust RAG pipelines, anchored by a modern FastAPI and PostgreSQL backend. The cloud_fullstack score indicates a minor gap in enterprise Azure deployment, though his Python and Redis proficiency mitigates this. This blend of architectural maturity and practical AI implementation makes him an immediate, low-risk asset for our engineering team.</t>
+          <t>Gourab Das (81.5/100) impressed with advanced rag with hybrid search and reranking alongside async fastapi backend architecture. Also notable: postgresql with orm / schema migrations. Depth spans Python, FastAPI, Django, Flask, PostgreSQL, Redis (cloud 14.0/15, GitHub 10.0/10). Activity: Veteran Builder (6.3 yrs on GitHub, 21 repos [12 original], 3 contributions in past year [0 commits]). 4 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1189,22 +1187,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Hari Shanker Sharma</t>
+          <t>Vivek Chimnani</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>harishankersharma648@gmail.com</t>
+          <t>vivekchimnani4231@gmail.com</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>+91 8801109700</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>candidate_41.pdf</t>
+          <t>candidate_44.pdf</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -1213,10 +1211,10 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>73.5</v>
+        <v>78.5</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>27</v>
@@ -1225,7 +1223,7 @@
         <v>14</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>3.5</v>
@@ -1237,25 +1235,25 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="T8" s="3" t="n">
         <v>0</v>
@@ -1268,12 +1266,12 @@
       </c>
       <c r="W8" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Redis, Docker, Kubernetes, AWS, LangChain, LangGraph, RAG, Qdrant, Embeddings, Vector Search, Openai, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, PostgreSQL, Redis, Docker, AWS, LangGraph, Claude, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd, Linux, Mongodb</t>
         </is>
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>Hari Shanker Sharma scored 73.5/100 (AI 29.0/40, Python 27.0/30, Cloud 14.0/15, GitHub 0.0/10), led by distributed task queues (celery/rabbitmq/kafka) and stateful multi-agent orchestration (langgraph/crewai/autogen) Backed by vector database retrieval (chromadb/faiss/pinecone/qdrant). Stack centers on Python, FastAPI, PostgreSQL, Redis. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: low or dormant public github activity. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>Vivek Chimnani scored 78.5/100 (AI 24.0/40, Python 27.0/30, Cloud 14.0/15, GitHub 10.0/10), led by stateful multi-agent orchestration (langgraph/crewai/autogen) and async fastapi backend architecture Backed by postgresql with orm / schema migrations. Stack centers on Python, FastAPI, PostgreSQL, Redis. GitHub: Veteran Builder (4.7 yrs on GitHub, 70 repos [25 original], 635 contributions in past year [0 commits]). 3 relevant Python/AI repositories identified. Watch-item: polishing production hardening. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -1283,22 +1281,22 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Sumaiya Sultana Shaik</t>
+          <t>Yash Maini</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>sultanasumaiya623@gmail.com</t>
+          <t>mainiyash2@gmail.com</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>+91 97015 28467</t>
+          <t>+91-8920028757</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>candidate_28.pdf</t>
+          <t>candidate_13.pdf</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1307,25 +1305,25 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>72.5</v>
+        <v>78</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>7.1</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1334,20 +1332,20 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>0</v>
+        <v>306</v>
       </c>
       <c r="T9" s="3" t="n">
         <v>0</v>
@@ -1356,16 +1354,16 @@
         <v>0</v>
       </c>
       <c r="V9" s="3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="W9" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Docker, GCP, LangChain, LangGraph, RAG, React, Typescript, Graphql, Rest Api, Pytest, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, GCP, AWS, LangChain, LangGraph, RAG, Faiss, Pinecone, Embeddings, Tool Calling, Openai, Claude, Pytorch, Tensorflow, Rest Api, Ci/Cd, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>Sumaiya Sultana Shaik demonstrates promising architectural instincts through stateful multi-agent orchestration using LangGraph and CrewAI, paired with a solid FastAPI and PostgreSQL backend. Her experience integrating RAG pipelines with Docker and GCP shows practical fullstack capability. However, her public GitHub activity is currently dormant or inaccessible due to API limits, obscuring her broader engineering depth. The primary gap is a lack of evidence for Redis caching or performance optimization. Despite these unknowns, her core AI backend skills align well with our intern needs, warranting a technical interview to validate her hands-on proficiency.</t>
+          <t>Yash Maini (78.0/100) impressed with postgresql with orm / schema migrations alongside docker containerization &amp; deployment. Also notable: gcp cloud deployment experience. Depth spans Python, FastAPI, Flask, PostgreSQL, Postgres, Docker (cloud 11.0/15, GitHub 10.0/10). Activity: Veteran Builder (3.8 yrs on GitHub, 47 repos [28 original], 306 contributions in past year [0 commits], 11 stars). 22 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1375,22 +1373,22 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Arjun Kumar</t>
+          <t>Kiran Naregal</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>roy.prajapat.143@gmail.com</t>
+          <t>kirnaregal7@gmail.com</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>+91-6396303191</t>
+          <t>9964923041</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>candidate_08.pdf</t>
+          <t>candidate_47.pdf</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1399,47 +1397,47 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>71.5</v>
+        <v>76.5</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>35</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J10" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Veteran Builder</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="Q10" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>8.279999999999999</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="inlineStr">
-        <is>
-          <t>Unverified (Rate Limited)</t>
-        </is>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="R10" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T10" s="3" t="n">
         <v>0</v>
@@ -1452,12 +1450,12 @@
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, PostgreSQL, AWS, LangChain, LangGraph, RAG, Embeddings, Gemini, Tensorflow, React, Next.js, Typescript, Javascript, Node.Js, Rest Api, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, Docker, AWS, LangChain, LangGraph, RAG, Openai, Anthropic, Claude, Ollama, Transformers, React, Next.js, Javascript, Node.Js, GIT, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>At 71.5/100, Arjun Kumar stands out through automated testing / ci/cd pipeline, complemented by observability and concurrency handling. Plus stateful multi-agent orchestration (langgraph/crewai/autogen) rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, AWS maps to AI 35.0 and Python 25.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
+          <t>Kiran Naregal (76.5/100) impressed with docker containerization &amp; deployment alongside cloud infrastructure (aws/azure). Also notable: full stack capability (react/next.js/typescript). Depth spans Python, FastAPI, Docker, AWS, LangChain, LangGraph (cloud 14.0/15, GitHub 6.0/10). Activity: Veteran Builder (5.4 yrs on GitHub, 8 repos [8 original], 3 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1467,22 +1465,22 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Kiran Naregal</t>
+          <t>Vaibhav Wakde</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>kirnaregal7@gmail.com</t>
+          <t>vaibhavwakde266@gmail.com</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>9964923041</t>
+          <t>+91-9307600143</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>candidate_47.pdf</t>
+          <t>candidate_33.pdf</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1491,25 +1489,27 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>70.5</v>
+        <v>75.5</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>8.76</v>
+        <v>3.5</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1518,20 +1518,20 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="T11" s="3" t="n">
         <v>0</v>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Docker, AWS, LangChain, LangGraph, RAG, Openai, Anthropic, Claude, Ollama, Transformers, React, Next.js, Javascript, Node.Js, GIT, SQL, Mongodb</t>
+          <t>Python, FastAPI, Flask, Docker, AWS, LangChain, LangGraph, LlamaIndex, RAG, ChromaDB, Weaviate, Tool Calling, Openai, Ollama, Transformers, Javascript, Pytest, GIT, SQL</t>
         </is>
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>Kiran Naregal scored 70.5/100 (AI 35.0/40, Python 20.0/30, Cloud 14.0/15, GitHub 0.0/10), led by observability and concurrency handling and stateful multi-agent orchestration (langgraph/crewai/autogen) Backed by embeddings-based retrieval system. Stack centers on Python, FastAPI, Docker, AWS. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>Vaibhav Wakde (75.5/100) impressed with cloud infrastructure (aws/azure) alongside strong public github footprint (veteran builder). Also notable: automated testing / ci/cd pipeline. Depth spans Python, FastAPI, Flask, Docker, AWS, LangChain (cloud 10.0/15, GitHub 10.0/10). Activity: Veteran Builder (3.5 yrs on GitHub, 10 repos [10 original], 12 contributions in past year [0 commits]). 4 relevant Python/AI repositories identified. Interview focus should be polishing production hardening, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -1559,22 +1559,22 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Vivek Chimnani</t>
+          <t>Arunima Saha</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>vivekchimnani4231@gmail.com</t>
+          <t>arunimasaha11@gmail.com</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91 9187656193</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>candidate_44.pdf</t>
+          <t>candidate_43.pdf</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1583,27 +1583,25 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>68.5</v>
+        <v>75.5</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1610,7 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Unlinked / Missing</t>
         </is>
       </c>
       <c r="P12" s="3" t="n">
@@ -1638,12 +1636,12 @@
       </c>
       <c r="W12" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Redis, Docker, AWS, LangGraph, Claude, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd, Linux, Mongodb</t>
+          <t>Python, FastAPI, PostgreSQL, Docker, Google Cloud, AWS, LangChain, LangGraph, RAG, Pinecone, Embeddings, Vector Search, Tool Calling, Openai, Gemini, Transformers, Rest Api, GIT, SQL</t>
         </is>
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>At 68.5/100, Vivek Chimnani stands out through automated testing / ci/cd pipeline, complemented by observability and concurrency handling. Plus stateful multi-agent orchestration (langgraph/crewai/autogen) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Redis, Docker maps to AI 24.0 and Python 27.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>Arunima’s portfolio reveals a sophisticated grasp of stateful multi-agent orchestration via LangGraph, a standout capability for complex AI workflows. Her backend architecture leverages Python, FastAPI, and PostgreSQL, demonstrating solid full-stack integration with Docker and cloud providers. However, the absence of a public GitHub profile hinders direct code review, while limited evidence of Redis caching or explicit pytest unit tests suggests a gap in production-readiness. This profile fits our SDE AI internship, requiring mentorship to bridge the delta between prototype complexity and rigorous, testable engineering standards.</t>
         </is>
       </c>
     </row>
@@ -1653,22 +1651,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Yash Maini</t>
+          <t>Abhinav Mishra</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>mainiyash2@gmail.com</t>
+          <t>abhinavmishra3322@gmail.com</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>+91-8920028757</t>
+          <t>+91 7701956829</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>candidate_13.pdf</t>
+          <t>candidate_10.pdf</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1677,25 +1675,27 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>68</v>
+        <v>73.5</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>8.609999999999999</v>
+        <v>3.5</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -1704,38 +1704,38 @@
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P13" s="3" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>0</v>
+        <v>4315</v>
       </c>
       <c r="T13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="W13" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, GCP, AWS, LangChain, LangGraph, RAG, Faiss, Pinecone, Embeddings, Tool Calling, Openai, Claude, Pytorch, Tensorflow, Rest Api, Ci/Cd, SQL, Mongodb</t>
+          <t>Python, FastAPI, PostgreSQL, Redis, Azure, LangGraph, RAG, Openai, React, Next.js, Typescript, Javascript, Node.Js, Ci/Cd</t>
         </is>
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t>Yash Maini scored 68.0/100 (AI 33.0/40, Python 22.0/30, Cloud 11.0/15, GitHub 0.0/10), led by automated testing / ci/cd pipeline and stateful multi-agent orchestration (langgraph/crewai/autogen) Backed by vector database retrieval (chromadb/faiss/pinecone/qdrant). Stack centers on Python, FastAPI, Flask, PostgreSQL. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>Abhinav’s portfolio reveals a seasoned builder with 3.4 years of consistent output, including 61 repositories and 4,315 contributions last year. His technical core is anchored in a modern Python backend using FastAPI, PostgreSQL, and Redis, complemented by sophisticated stateful multi-agent orchestration via LangGraph. This combination of robust API design and advanced RAG implementation demonstrates rare depth for an intern. With no major gaps identified, his proven engineering discipline and broad Azure experience make him an immediate, high-value addition to our AI infrastructure team.</t>
         </is>
       </c>
     </row>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Prajwal A S</t>
+          <t>Jyandeep Baishya</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>prajwalas8999@gmail.com</t>
+          <t>craftzyan@gmail.com</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>6002590335</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>candidate_22.pdf</t>
+          <t>candidate_07.pdf</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1769,27 +1769,25 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M14" s="2" t="n">
+        <v>7.1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1798,20 +1796,20 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Active Builder</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P14" s="3" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="R14" s="3" t="n">
         <v>29</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>44</v>
+        <v>490</v>
       </c>
       <c r="T14" s="3" t="n">
         <v>0</v>
@@ -1820,16 +1818,16 @@
         <v>0</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W14" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Ollama, React, Javascript, Rest Api, GIT, Linux, SQL</t>
+          <t>Python, FastAPI, Redis, LangChain, LangGraph, RAG, ChromaDB, Tool Calling, React, Next.js, Typescript, Node.Js</t>
         </is>
       </c>
       <c r="X14" s="3" t="inlineStr">
         <is>
-          <t>At 68.0/100, Prajwal A S stands out through embeddings-based retrieval system, complemented by async fastapi backend architecture. Plus postgresql with orm / schema migrations rounds out the build. Core evidence in Python, FastAPI, Flask, PostgreSQL, LangChain maps to AI 31.0 and Python 25.0 bands. GitHub profile: Active Builder (2.9 yrs on GitHub, 32 repos [29 original], 44 contributions in past year [0 commits]). 13 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
+          <t>Jyandeep Baishya’s profile reveals a committed builder, evidenced by 45 repositories and 490 annual contributions. His technical foundation is solid, leveraging Python, FastAPI, and Redis to construct robust backend systems. He effectively integrates LangChain, LangGraph, and ChromaDB to deploy RAG pipelines and multi-agent workflows. While his GitHub history demonstrates consistent, original work, the absence of explicit testing frameworks like pytest remains a notable gap. This candidate is ready to contribute to our AI infrastructure, requiring mentorship to rigorize quality assurance practices during the internship.</t>
         </is>
       </c>
     </row>
@@ -1839,22 +1837,22 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Jyandeep Baishya</t>
+          <t>Nevil Jasmin Mehta</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>craftzyan@gmail.com</t>
+          <t>nevilmehta5@gmail.com</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>6002590335</t>
+          <t>+91-8347062282</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>candidate_07.pdf</t>
+          <t>candidate_50.pdf</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1863,25 +1861,25 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>63</v>
+        <v>70.5</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>7.1</v>
+        <v>9.56</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1890,20 +1888,20 @@
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P15" s="3" t="n">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="T15" s="3" t="n">
         <v>0</v>
@@ -1916,12 +1914,12 @@
       </c>
       <c r="W15" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Redis, LangChain, LangGraph, RAG, ChromaDB, Tool Calling, React, Next.js, Typescript, Node.Js</t>
+          <t>Python, FastAPI, Django, Flask, PostgreSQL, Redis, Docker, AWS, RAG, Qdrant, Embeddings, React, Javascript, Celery, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X15" s="3" t="inlineStr">
         <is>
-          <t>At 63.0/100, Jyandeep Baishya stands out through cloud infrastructure (aws/azure), complemented by full stack capability (react/next.js/typescript). Plus stateful multi-agent orchestration (langgraph/crewai/autogen) rounds out the build. Core evidence in Python, FastAPI, Redis, LangChain, LangGraph maps to AI 33.0 and Python 22.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>At 70.5/100, Nevil Jasmin Mehta stands out through async fastapi backend architecture, complemented by postgresql with orm / schema migrations. Plus redis caching / in-memory store rounds out the build. Core evidence in Python, FastAPI, Django, Flask, PostgreSQL maps to AI 18.0 and Python 27.0 bands. GitHub profile: Veteran Builder (6.9 yrs on GitHub, 19 repos [19 original], 250 contributions in past year [0 commits]). 15 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -1931,22 +1929,22 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>M Sai Kushith</t>
+          <t>Krishan Kant</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>msaikushith718@gmail.com</t>
+          <t>krishankantptu@gmail.com</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>+91-7842732706</t>
+          <t>+91-6204142591</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>candidate_06.pdf</t>
+          <t>candidate_09.pdf</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1955,49 +1953,47 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Veteran Builder</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K16" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="L16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O16" s="3" t="inlineStr">
-        <is>
-          <t>Active Builder</t>
-        </is>
-      </c>
-      <c r="P16" s="3" t="n">
-        <v>1.3</v>
-      </c>
       <c r="Q16" s="3" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="T16" s="3" t="n">
         <v>0</v>
@@ -2006,16 +2002,16 @@
         <v>0</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W16" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, PostgreSQL, LangChain, LangGraph, RAG, React, Typescript, GIT, Linux, SQL, Java</t>
+          <t>Python, PostgreSQL, Redis, Docker, LangChain, RAG, Vector Search, Openai, React, Typescript, Javascript, Kafka, GIT, SQL, Mongodb, Java, Spring Boot</t>
         </is>
       </c>
       <c r="X16" s="3" t="inlineStr">
         <is>
-          <t>At 61.0/100, M Sai Kushith stands out through full stack capability (react/next.js/typescript), complemented by stateful multi-agent orchestration (langgraph/crewai/autogen). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, FastAPI, Django, PostgreSQL, LangChain maps to AI 31.0 and Python 20.0 bands. GitHub profile: Active Builder (1.3 yrs on GitHub, 4 repos [4 original], 1 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
+          <t>Krishan’s four-year GitHub tenure reveals a builder’s mindset, anchored by two relevant Python/AI repositories. His strongest signal is an agentic workflow leveraging LangChain and OpenAI for function calling, paired with a robust embeddings-based retrieval system using PostgreSQL and Redis. While the stack is solid, the absence of explicit pytest unit tests hints at a need for rigorous engineering discipline. This gap, however, is exactly what our internship program targets, offering him the structured mentorship to refine his RAG pipelines into production-grade, testable code.</t>
         </is>
       </c>
     </row>
@@ -2025,22 +2021,22 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Krishan Kant</t>
+          <t>Prajwal A S</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>krishankantptu@gmail.com</t>
+          <t>prajwalas8999@gmail.com</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>+91-6204142591</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>candidate_09.pdf</t>
+          <t>candidate_22.pdf</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2049,25 +2045,27 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>25</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>7.33</v>
+        <v>0</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -2076,20 +2074,20 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P17" s="3" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="S17" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="T17" s="3" t="n">
         <v>0</v>
@@ -2102,12 +2100,12 @@
       </c>
       <c r="W17" s="3" t="inlineStr">
         <is>
-          <t>Python, PostgreSQL, Redis, Docker, LangChain, RAG, Vector Search, Openai, React, Typescript, Javascript, Kafka, GIT, SQL, Mongodb, Java, Spring Boot</t>
+          <t>Python, FastAPI, Flask, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Ollama, React, Javascript, Rest Api, GIT, Linux, SQL</t>
         </is>
       </c>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t>At 61.0/100, Krishan Kant stands out through distributed task queues (celery/rabbitmq/kafka), complemented by observability and concurrency handling. Plus agentic workflow with tool/function calling rounds out the build. Core evidence in Python, PostgreSQL, Redis, Docker, LangChain maps to AI 23.0 and Python 25.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>At 68.0/100, Prajwal A S stands out through embeddings-based retrieval system, complemented by async fastapi backend architecture. Plus postgresql with orm / schema migrations rounds out the build. Core evidence in Python, FastAPI, Flask, PostgreSQL, LangChain maps to AI 31.0 and Python 25.0 bands. GitHub profile: Active Builder (2.9 yrs on GitHub, 32 repos [29 original], 44 contributions in past year [0 commits]). 13 relevant Python/AI repositories identified. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -2117,22 +2115,22 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Nevil Jasmin Mehta</t>
+          <t>Priyanshu Kumar</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>nevilmehta5@gmail.com</t>
+          <t>krpriyanshu2805@gmail.com</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>+91-8347062282</t>
+          <t>+91 8210008947</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>candidate_50.pdf</t>
+          <t>candidate_16.pdf</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -2141,25 +2139,25 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>60.5</v>
+        <v>63</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="L18" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>9.56</v>
+        <v>8</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -2168,20 +2166,20 @@
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P18" s="3" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T18" s="3" t="n">
         <v>0</v>
@@ -2194,12 +2192,12 @@
       </c>
       <c r="W18" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, Flask, PostgreSQL, Redis, Docker, AWS, RAG, Qdrant, Embeddings, React, Javascript, Celery, SQL, Mongodb, Java</t>
+          <t>Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG, Pinecone, Embeddings, Tool Calling, React, Javascript, Node.Js, Kafka, GIT, Mongodb</t>
         </is>
       </c>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t>Nevil Jasmin Mehta (60.5/100) impressed with vector database retrieval (chromadb/faiss/pinecone/qdrant) alongside async fastapi backend architecture. Also notable: postgresql with orm / schema migrations. Depth spans Python, FastAPI, Django, Flask, PostgreSQL, Redis (cloud 14.0/15, GitHub 0.0/10). Activity: GitHub API rate limit exceeded; skipped enrichment. Interview focus should be low or dormant public github activity, but overall internship readiness is high.</t>
+          <t>Priyanshu Kumar (63.0/100) impressed with full stack capability (react/next.js/typescript) alongside strong public github footprint (veteran builder). Also notable: distributed task queues (celery/rabbitmq/kafka). Depth spans Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG (cloud 4.0/15, GitHub 7.5/10). Activity: Veteran Builder (3.3 yrs on GitHub, 13 repos [9 original], 5 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -2209,22 +2207,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Thejeshwaar Paasila</t>
+          <t>P V Jayavardhana Sai</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>thejeshwaarp@gmail.com</t>
+          <t>pvjayavardhan6@gmail.com</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>+91 6303204136</t>
+          <t>+91 99663 46173</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>candidate_26.pdf</t>
+          <t>candidate_19.pdf</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2233,50 +2231,48 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>59.5</v>
+        <v>62</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>8.6</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Emerging Developer</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P19" s="3" t="n">
-        <v>2.3</v>
+        <v>3.7</v>
       </c>
       <c r="Q19" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="S19" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="R19" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="S19" s="3" t="n">
-        <v>10</v>
-      </c>
       <c r="T19" s="3" t="n">
         <v>0</v>
       </c>
@@ -2284,16 +2280,16 @@
         <v>0</v>
       </c>
       <c r="V19" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W19" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, PostgreSQL, Docker, Google Cloud, RAG, Openai, Gemini, Claude, Transformers, React, Next.js, Typescript, Javascript, Node.Js, GIT, Ci/Cd, Linux, SQL, Mongodb</t>
+          <t>Python, Flask, Docker, AWS, RAG, Ollama, Transformers, Pytorch, Tensorflow, React, Javascript, GIT, SQL, Java</t>
         </is>
       </c>
       <c r="X19" s="3" t="inlineStr">
         <is>
-          <t>At 59.5/100, Thejeshwaar Paasila stands out through modern python backend framework (fastapi/django), complemented by postgresql with orm / schema migrations. Plus docker containerization &amp; deployment rounds out the build. Core evidence in Python, Flask, PostgreSQL, Docker, Google Cloud maps to AI 16.0 and Python 20.0 bands. GitHub profile: Emerging Developer (2.3 yrs on GitHub, 3 repos [2 original], 10 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
+          <t>P V Jayavardhana Sai (62.0/100) impressed with ai evaluation pipeline (ragas/langsmith/trulens) alongside modern python backend framework (fastapi/django). Also notable: docker containerization &amp; deployment. Depth spans Python, Flask, Docker, AWS, RAG, Ollama (cloud 14.0/15, GitHub 7.5/10). Activity: Veteran Builder (3.7 yrs on GitHub, 8 repos [8 original], 3 contributions in past year [0 commits], 1 stars). 5 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -2303,22 +2299,22 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Vivek Shekhawat</t>
+          <t>M Sai Kushith</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>vivekshekhawatofficial1592002@gmail.com</t>
+          <t>msaikushith718@gmail.com</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>+91-7734911626</t>
+          <t>+91-7842732706</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>candidate_39.pdf</t>
+          <t>candidate_06.pdf</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2327,44 +2323,46 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J20" s="3" t="n">
         <v>4</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>9.140000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Veteran Builder</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P20" s="3" t="n">
-        <v>4.1</v>
+        <v>1.3</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="S20" s="3" t="n">
         <v>1</v>
@@ -2380,12 +2378,12 @@
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
-          <t>Python, Django, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Vector Search, Ollama, React, Next.js, Javascript, Node.Js, GIT, SQL, Java</t>
+          <t>Python, FastAPI, Django, PostgreSQL, LangChain, LangGraph, RAG, React, Typescript, GIT, Linux, SQL, Java</t>
         </is>
       </c>
       <c r="X20" s="3" t="inlineStr">
         <is>
-          <t>Vivek Shekhawat scored 59.0/100 (AI 27.0/40, Python 23.0/30, Cloud 4.0/15, GitHub 3.5/10), led by postgresql with orm / schema migrations and full stack capability (react/next.js/typescript) Backed by observability and concurrency handling. Stack centers on Python, Django, PostgreSQL, LangChain. GitHub: Veteran Builder (4.1 yrs on GitHub, 15 repos [0 original], 1 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Watch-item: no explicit testing (pytest/unit tests) mentioned. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>M Sai Kushith’s portfolio reveals a promising trajectory, anchored by one relevant Python/AI repository demonstrating RAG capabilities via LangChain and LangGraph. While the backend infrastructure is minimal, the integration of PostgreSQL suggests foundational database literacy. However, the 1.3-year GitHub history with only four total repositories indicates limited sustained engineering output. The absence of explicit testing practices or Redis caching remains a critical gap. Despite these shortcomings, the niche focus on retrieval systems warrants a junior internship to build robust backend discipline.</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2393,22 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Pavani A</t>
+          <t>Thejeshwaar Paasila</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>pavani10112004@gmail.com</t>
+          <t>thejeshwaarp@gmail.com</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>+919742542200</t>
+          <t>+91 6303204136</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>candidate_38.pdf</t>
+          <t>candidate_26.pdf</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2419,47 +2417,49 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>58</v>
+        <v>59.5</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>20</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="M21" s="2" t="n">
-        <v>9.710000000000001</v>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Active Builder</t>
+          <t>Emerging Developer</t>
         </is>
       </c>
       <c r="P21" s="3" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S21" s="3" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="T21" s="3" t="n">
         <v>0</v>
@@ -2472,12 +2472,12 @@
       </c>
       <c r="W21" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Django, Flask, PostgreSQL, Docker, Tensorflow, React, Next.js, Javascript, GIT, Ci/Cd, SQL, Mongodb, Java</t>
+          <t>Python, Flask, PostgreSQL, Docker, Google Cloud, RAG, Openai, Gemini, Claude, Transformers, React, Next.js, Typescript, Javascript, Node.Js, GIT, Ci/Cd, Linux, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X21" s="3" t="inlineStr">
         <is>
-          <t>At 58.0/100, Pavani A stands out through postgresql with orm / schema migrations, complemented by docker containerization &amp; deployment. Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, Django, Flask, PostgreSQL maps to AI 20.0 and Python 20.0 bands. GitHub profile: Active Builder (1.9 yrs on GitHub, 16 repos [0 original], 19 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
+          <t>At 59.5/100, Thejeshwaar Paasila stands out through modern python backend framework (fastapi/django), complemented by postgresql with orm / schema migrations. Plus docker containerization &amp; deployment rounds out the build. Core evidence in Python, Flask, PostgreSQL, Docker, Google Cloud maps to AI 16.0 and Python 20.0 bands. GitHub profile: Emerging Developer (2.3 yrs on GitHub, 3 repos [2 original], 10 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -2487,22 +2487,22 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Aditi Kala</t>
+          <t>Raj Thumar</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>aditi25.kala@gmail.com</t>
+          <t>thumarraj999@gmail.com</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>+91-8368407039</t>
+          <t>+91 9104382983</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>candidate_37.pdf</t>
+          <t>candidate_40.pdf</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2511,22 +2511,22 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>58</v>
+        <v>59.5</v>
       </c>
       <c r="H22" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="J22" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="I22" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="J22" s="3" t="n">
-        <v>15</v>
-      </c>
       <c r="K22" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
@@ -2544,34 +2544,34 @@
         </is>
       </c>
       <c r="P22" s="3" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>567</v>
+        <v>7</v>
       </c>
       <c r="T22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="V22" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W22" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, Google Cloud, Gemini, Pytorch, Tensorflow, React, Node.Js, GIT, SQL, Mongodb, Java</t>
+          <t>Python, Flask, PostgreSQL, Redis, Docker, AWS, RAG, Openai, Gemini, React, Typescript, Javascript, Node.Js, Graphql, Kafka, Mongodb</t>
         </is>
       </c>
       <c r="X22" s="3" t="inlineStr">
         <is>
-          <t>Aditi Kala scored 58.0/100 (AI 14.0/40, Python 23.0/30, Cloud 15.0/15, GitHub 6.0/10), led by basic agent implementation and embeddings-based retrieval system Backed by modern python backend framework (fastapi/django). Stack centers on Python, FastAPI, Flask, PostgreSQL. GitHub: Veteran Builder (3.5 yrs on GitHub, 53 repos [0 original], 567 contributions in past year [0 commits, 27 PRs]). 0 relevant Python/AI repositories identified. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>At 59.5/100, Raj Thumar stands out through modern python backend framework (fastapi/django), complemented by postgresql with orm / schema migrations. Plus redis caching / in-memory store rounds out the build. Core evidence in Python, Flask, PostgreSQL, Redis, Docker maps to AI 12.0 and Python 25.0 bands. GitHub profile: Veteran Builder (3.3 yrs on GitHub, 10 repos [10 original], 7 contributions in past year [0 commits], 2 stars). 0 relevant Python/AI repositories identified. Growth edge to probe in interview: polishing production hardening.</t>
         </is>
       </c>
     </row>
@@ -2581,22 +2581,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Priyanshu Kumar</t>
+          <t>Shubhanshu Navadiya</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>krpriyanshu2805@gmail.com</t>
+          <t>subhnavadiya@gmail.com</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>+91 8210008947</t>
+          <t>+91 9031132507</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>candidate_16.pdf</t>
+          <t>candidate_12.pdf</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2605,47 +2605,47 @@
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>55.5</v>
+        <v>59</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Veteran Builder</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O23" s="3" t="inlineStr">
-        <is>
-          <t>Unverified (Rate Limited)</t>
-        </is>
-      </c>
-      <c r="P23" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="Q23" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="S23" s="3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="T23" s="3" t="n">
         <v>0</v>
@@ -2654,16 +2654,16 @@
         <v>0</v>
       </c>
       <c r="V23" s="3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="W23" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, LangChain, LangGraph, RAG, Pinecone, Embeddings, Tool Calling, React, Javascript, Node.Js, Kafka, GIT, Mongodb</t>
+          <t>Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant, Weaviate, Embeddings, Openai, Gemini, Ollama, Transformers, Pytorch, GIT, SQL</t>
         </is>
       </c>
       <c r="X23" s="3" t="inlineStr">
         <is>
-          <t>Priyanshu Kumar scored 55.5/100 (AI 28.0/40, Python 22.0/30, Cloud 4.0/15, GitHub 0.0/10), led by stateful multi-agent orchestration (langgraph/crewai/autogen) and vector database retrieval (chromadb/faiss/pinecone/qdrant) Backed by async fastapi backend architecture. Stack centers on Python, FastAPI, PostgreSQL, LangChain. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>Shubhanshu Navadiya (59.0/100) impressed with automated testing / ci/cd pipeline alongside stateful multi-agent orchestration (langgraph/crewai/autogen). Also notable: vector database retrieval (chromadb/faiss/pinecone/qdrant). Depth spans Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant (cloud 0.0/15, GitHub 8.0/10). Activity: Veteran Builder (4.0 yrs on GitHub, 25 repos [7 original], 43 contributions in past year [0 commits], 21 stars). 14 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -2673,22 +2673,22 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>P V Jayavardhana Sai</t>
+          <t>Vivek Shekhawat</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>pvjayavardhan6@gmail.com</t>
+          <t>vivekshekhawatofficial1592002@gmail.com</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>+91 99663 46173</t>
+          <t>+91-7734911626</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>candidate_19.pdf</t>
+          <t>candidate_39.pdf</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2697,25 +2697,25 @@
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>54.5</v>
+        <v>59</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="L24" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>8.6</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -2724,20 +2724,20 @@
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P24" s="3" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="R24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T24" s="3" t="n">
         <v>0</v>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, Docker, AWS, RAG, Ollama, Transformers, Pytorch, Tensorflow, React, Javascript, GIT, SQL, Java</t>
+          <t>Python, Django, PostgreSQL, LangChain, LangGraph, RAG, Embeddings, Vector Search, Ollama, React, Next.js, Javascript, Node.Js, GIT, SQL, Java</t>
         </is>
       </c>
       <c r="X24" s="3" t="inlineStr">
         <is>
-          <t>At 54.5/100, P V Jayavardhana Sai stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, Flask, Docker, AWS, RAG maps to AI 22.0 and Python 17.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>Vivek Shekhawat scored 59.0/100 (AI 27.0/40, Python 23.0/30, Cloud 4.0/15, GitHub 3.5/10), led by postgresql with orm / schema migrations and full stack capability (react/next.js/typescript) Backed by observability and concurrency handling. Stack centers on Python, Django, PostgreSQL, LangChain. GitHub: Veteran Builder (4.1 yrs on GitHub, 15 repos [0 original], 1 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Watch-item: no explicit testing (pytest/unit tests) mentioned. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -2765,22 +2765,22 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Raj Thumar</t>
+          <t>Aditi Kala</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>thumarraj999@gmail.com</t>
+          <t>aditi25.kala@gmail.com</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>+91 9104382983</t>
+          <t>+91-8368407039</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>candidate_40.pdf</t>
+          <t>candidate_37.pdf</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -2789,67 +2789,67 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>54.5</v>
+        <v>58</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Veteran Builder</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="inlineStr">
-        <is>
-          <t>Unverified (Rate Limited)</t>
-        </is>
-      </c>
-      <c r="P25" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="Q25" s="3" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="R25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S25" s="3" t="n">
-        <v>0</v>
+        <v>567</v>
       </c>
       <c r="T25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U25" s="3" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="V25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W25" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, PostgreSQL, Redis, Docker, AWS, RAG, Openai, Gemini, React, Typescript, Javascript, Node.Js, Graphql, Kafka, Mongodb</t>
+          <t>Python, FastAPI, Flask, PostgreSQL, Postgres, Docker, Google Cloud, Gemini, Pytorch, Tensorflow, React, Node.Js, GIT, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X25" s="3" t="inlineStr">
         <is>
-          <t>At 54.5/100, Raj Thumar stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, Flask, PostgreSQL, Redis, Docker maps to AI 12.0 and Python 25.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>Aditi Kala scored 58.0/100 (AI 14.0/40, Python 23.0/30, Cloud 15.0/15, GitHub 6.0/10), led by basic agent implementation and embeddings-based retrieval system Backed by modern python backend framework (fastapi/django). Stack centers on Python, FastAPI, Flask, PostgreSQL. GitHub: Veteran Builder (3.5 yrs on GitHub, 53 repos [0 original], 567 contributions in past year [0 commits, 27 PRs]). 0 relevant Python/AI repositories identified. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -2859,22 +2859,22 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Harsha A</t>
+          <t>Pavani A</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>harshaarun2608@gmail.com</t>
+          <t>pavani10112004@gmail.com</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>+91-9113869665</t>
+          <t>+919742542200</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>candidate_15.pdf</t>
+          <t>candidate_38.pdf</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>20</v>
@@ -2892,38 +2892,38 @@
         <v>20</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>7.55</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>Unlinked / Missing</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P26" s="3" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S26" s="3" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="T26" s="3" t="n">
         <v>0</v>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="W26" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Docker, Azure, Tensorflow, React, Javascript, Node.Js, SQL, Java</t>
+          <t>Python, FastAPI, Django, Flask, PostgreSQL, Docker, Tensorflow, React, Next.js, Javascript, GIT, Ci/Cd, SQL, Mongodb, Java</t>
         </is>
       </c>
       <c r="X26" s="3" t="inlineStr">
         <is>
-          <t>At 54.0/100, Harsha A stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Docker, Azure maps to AI 20.0 and Python 20.0 bands. GitHub profile: No public GitHub profile provided. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
+          <t>At 58.0/100, Pavani A stands out through postgresql with orm / schema migrations, complemented by docker containerization &amp; deployment. Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, Django, Flask, PostgreSQL maps to AI 20.0 and Python 20.0 bands. GitHub profile: Active Builder (1.9 yrs on GitHub, 16 repos [0 original], 19 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -2951,22 +2951,22 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Shubhanshu Navadiya</t>
+          <t>Aswin Raj R</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>subhnavadiya@gmail.com</t>
+          <t>aswinrajr12@gmail.com</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>+91 9031132507</t>
+          <t>+91-7994013148</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>candidate_12.pdf</t>
+          <t>candidate_49.pdf</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2975,25 +2975,27 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>17</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>8.1</v>
+        <v>0</v>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
@@ -3002,20 +3004,20 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P27" s="3" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="S27" s="3" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="T27" s="3" t="n">
         <v>0</v>
@@ -3028,12 +3030,12 @@
       </c>
       <c r="W27" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant, Weaviate, Embeddings, Openai, Gemini, Ollama, Transformers, Pytorch, GIT, SQL</t>
+          <t>Python, AWS, LangChain, RAG, Openai, Tensorflow, React, Javascript, Node.Js, GIT, Linux, SQL, Mongodb, Java, Spring Boot</t>
         </is>
       </c>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t>Shubhanshu Navadiya (51.0/100) impressed with stateful multi-agent orchestration (langgraph/crewai/autogen) alongside vector database retrieval (chromadb/faiss/pinecone/qdrant). Also notable: ai evaluation pipeline (ragas/langsmith/trulens). Depth spans Python, FastAPI, LangChain, LlamaIndex, RAG, Qdrant (cloud 0.0/15, GitHub 0.0/10). Activity: GitHub API rate limit exceeded; skipped enrichment. Interview focus should be low or dormant public github activity, but overall internship readiness is high.</t>
+          <t>Aswin Raj R (58.0/100) impressed with agentic workflow with tool/function calling alongside embeddings-based retrieval system. Also notable: cloud infrastructure (aws/azure). Depth spans Python, AWS, LangChain, RAG, Openai, Tensorflow (cloud 8.0/15, GitHub 10.0/10). Activity: Active Builder (1.6 yrs on GitHub, 13 repos [13 original], 69 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be no explicit testing (pytest/unit tests) mentioned, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -3043,22 +3045,22 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Aswin Raj R</t>
+          <t>Harsha A</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>aswinrajr12@gmail.com</t>
+          <t>harshaarun2608@gmail.com</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>+91-7994013148</t>
+          <t>+91-9113869665</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>candidate_49.pdf</t>
+          <t>candidate_15.pdf</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -3067,16 +3069,16 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="K28" s="3" t="n">
         <v>0</v>
@@ -3084,19 +3086,17 @@
       <c r="L28" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M28" s="2" t="n">
+        <v>7.55</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Unlinked / Missing</t>
         </is>
       </c>
       <c r="P28" s="3" t="n">
@@ -3122,12 +3122,12 @@
       </c>
       <c r="W28" s="3" t="inlineStr">
         <is>
-          <t>Python, AWS, LangChain, RAG, Openai, Tensorflow, React, Javascript, Node.Js, GIT, Linux, SQL, Mongodb, Java, Spring Boot</t>
+          <t>Python, FastAPI, PostgreSQL, Docker, Azure, Tensorflow, React, Javascript, Node.Js, SQL, Java</t>
         </is>
       </c>
       <c r="X28" s="3" t="inlineStr">
         <is>
-          <t>Aswin Raj R scored 48.0/100 (AI 23.0/40, Python 17.0/30, Cloud 8.0/15, GitHub 0.0/10), led by embeddings-based retrieval system and cloud infrastructure (aws/azure) Backed by full stack capability (react/next.js/typescript). Stack centers on Python, AWS, LangChain, RAG. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>At 54.0/100, Harsha A stands out through docker containerization &amp; deployment, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Docker, Azure maps to AI 20.0 and Python 20.0 bands. GitHub profile: No public GitHub profile provided. Growth edge to probe in interview: no explicit testing (pytest/unit tests) mentioned.</t>
         </is>
       </c>
     </row>
@@ -3137,22 +3137,22 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Annisha S</t>
+          <t>Higher Secondary Science Pcmb</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>annishasaravanan83@gmail.com</t>
+          <t>manojkumar.k.r0904@gmail.com</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>9361112081</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>candidate_23.pdf</t>
+          <t>candidate_21.pdf</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3161,25 +3161,25 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>8.720000000000001</v>
+        <v>7.65</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
@@ -3188,20 +3188,20 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Emerging Developer</t>
         </is>
       </c>
       <c r="P29" s="3" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T29" s="3" t="n">
         <v>0</v>
@@ -3214,12 +3214,12 @@
       </c>
       <c r="W29" s="3" t="inlineStr">
         <is>
-          <t>Python, FastAPI, PostgreSQL, Azure, LangGraph, Openai, React, GIT, SQL, Mongodb</t>
+          <t>Python, Flask, Pytorch, Tensorflow, React, GIT, SQL, Java</t>
         </is>
       </c>
       <c r="X29" s="3" t="inlineStr">
         <is>
-          <t>At 43.0/100, Annisha S stands out through postgresql with orm / schema migrations, complemented by cloud infrastructure (aws/azure). Plus full stack capability (react/next.js/typescript) rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Azure, LangGraph maps to AI 15.0 and Python 20.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>Higher Secondary Science Pcmb (47.0/100) impressed with ai evaluation pipeline (ragas/langsmith/trulens) alongside modern python backend framework (fastapi/django). Also notable: full stack capability (react/next.js/typescript). Depth spans Python, Flask, Pytorch, Tensorflow, React, GIT (cloud 4.0/15, GitHub 6.0/10). Activity: Emerging Developer (1.9 yrs on GitHub, 1 repos [1 original], 3 contributions in past year [0 commits]). 1 relevant Python/AI repositories identified. Interview focus should be no explicit testing (pytest/unit tests) mentioned, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -3229,22 +3229,22 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Atul Kumar</t>
+          <t>Annisha S</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>atulofficial02@gmail.com</t>
+          <t>annishasaravanan83@gmail.com</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>+91-9368449979</t>
+          <t>9361112081</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>candidate_25.pdf</t>
+          <t>candidate_23.pdf</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3253,27 +3253,25 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="M30" s="2" t="n">
+        <v>8.720000000000001</v>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
@@ -3282,20 +3280,20 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Active Builder</t>
+          <t>Active Developer</t>
         </is>
       </c>
       <c r="P30" s="3" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="R30" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="S30" s="3" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="T30" s="3" t="n">
         <v>0</v>
@@ -3308,12 +3306,12 @@
       </c>
       <c r="W30" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, GCP, Google Cloud, Gemini, Rest Api, GIT, SQL</t>
+          <t>Python, FastAPI, PostgreSQL, Azure, LangGraph, Openai, React, GIT, SQL, Mongodb</t>
         </is>
       </c>
       <c r="X30" s="3" t="inlineStr">
         <is>
-          <t>Atul Kumar (42.0/100) impressed with embeddings-based retrieval system alongside modern python backend framework (fastapi/django). Also notable: gcp cloud deployment experience. Depth spans Python, Flask, GCP, Google Cloud, Gemini, Rest Api (cloud 5.0/15, GitHub 8.0/10). Activity: Active Builder (1.7 yrs on GitHub, 9 repos [9 original], 42 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
+          <t>At 44.0/100, Annisha S stands out through stateful multi-agent orchestration (langgraph/crewai/autogen), complemented by modern python backend framework (fastapi/django). Plus postgresql with orm / schema migrations rounds out the build. Core evidence in Python, FastAPI, PostgreSQL, Azure, LangGraph maps to AI 15.0 and Python 20.0 bands. GitHub profile: Active Developer (2.3 yrs on GitHub, 4 repos [3 original], 0 contributions in past year [0 commits]). 0 relevant Python/AI repositories identified. Growth edge to probe in interview: limited redis or backend caching evidence.</t>
         </is>
       </c>
     </row>
@@ -3323,22 +3321,22 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Higher Secondary Science Pcmb</t>
+          <t>Dornipadu Karthika Chaitrika</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>manojkumar.k.r0904@gmail.com</t>
+          <t>dornipadukarthi@gmail.com</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+91-9014209602</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>candidate_21.pdf</t>
+          <t>candidate_24.pdf</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -3347,47 +3345,47 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H31" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>Active Builder</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="Q31" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="I31" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="J31" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="K31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>7.65</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O31" s="3" t="inlineStr">
-        <is>
-          <t>Unverified (Rate Limited)</t>
-        </is>
-      </c>
-      <c r="P31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="R31" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="S31" s="3" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="T31" s="3" t="n">
         <v>0</v>
@@ -3396,16 +3394,16 @@
         <v>0</v>
       </c>
       <c r="V31" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W31" s="3" t="inlineStr">
         <is>
-          <t>Python, Flask, Pytorch, Tensorflow, React, GIT, SQL, Java</t>
+          <t>Python, Django, Flask, RAG, Embeddings, Gemini, Javascript</t>
         </is>
       </c>
       <c r="X31" s="3" t="inlineStr">
         <is>
-          <t>At 41.0/100, Higher Secondary Science Pcmb stands out through modern python backend framework (fastapi/django), complemented by full stack capability (react/next.js/typescript). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, Flask, Pytorch, Tensorflow, React maps to AI 20.0 and Python 17.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>Dornipadu Karthika Chaitrika scored 44.0/100 (AI 23.0/40, Python 12.0/30, Cloud 0.0/15, GitHub 9.0/10), led by embeddings-based retrieval system and modern python backend framework (fastapi/django) Backed by strong public github footprint (active builder). Stack centers on Python, Django, Flask, RAG. GitHub: Active Builder (2.6 yrs on GitHub, 20 repos [20 original], 135 contributions in past year [0 commits], 1 stars). 12 relevant Python/AI repositories identified. Watch-item: no explicit testing (pytest/unit tests) mentioned. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -3415,22 +3413,22 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Dornipadu Karthika Chaitrika</t>
+          <t>Atul Kumar</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>dornipadukarthi@gmail.com</t>
+          <t>atulofficial02@gmail.com</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>+91-9014209602</t>
+          <t>+91-9368449979</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>candidate_24.pdf</t>
+          <t>candidate_25.pdf</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -3439,25 +3437,27 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M32" s="2" t="n">
-        <v>8.43</v>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
@@ -3466,20 +3466,20 @@
       </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Active Builder</t>
         </is>
       </c>
       <c r="P32" s="3" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="R32" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="S32" s="3" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="T32" s="3" t="n">
         <v>0</v>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="W32" s="3" t="inlineStr">
         <is>
-          <t>Python, Django, Flask, RAG, Embeddings, Gemini, Javascript</t>
+          <t>Python, Flask, GCP, Google Cloud, Gemini, Rest Api, GIT, SQL</t>
         </is>
       </c>
       <c r="X32" s="3" t="inlineStr">
         <is>
-          <t>Dornipadu Karthika Chaitrika scored 35.0/100 (AI 23.0/40, Python 12.0/30, Cloud 0.0/15, GitHub 0.0/10), led by basic agent implementation and embeddings-based retrieval system Backed by modern python backend framework (fastapi/django). Stack centers on Python, Django, Flask, RAG. GitHub: GitHub API rate limit exceeded; skipped enrichment. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
+          <t>Atul Kumar (42.0/100) impressed with embeddings-based retrieval system alongside modern python backend framework (fastapi/django). Also notable: gcp cloud deployment experience. Depth spans Python, Flask, GCP, Google Cloud, Gemini, Rest Api (cloud 5.0/15, GitHub 8.0/10). Activity: Active Builder (1.7 yrs on GitHub, 9 repos [9 original], 42 contributions in past year [0 commits]). 7 relevant Python/AI repositories identified. Interview focus should be limited redis or backend caching evidence, but overall internship readiness is high.</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H33" s="3" t="n">
         <v>7</v>
@@ -3543,7 +3543,7 @@
         <v>4</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L33" s="3" t="n">
         <v>0</v>
@@ -3558,20 +3558,20 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Unverified (Rate Limited)</t>
+          <t>Veteran Builder</t>
         </is>
       </c>
       <c r="P33" s="3" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="R33" s="3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="S33" s="3" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="T33" s="3" t="n">
         <v>0</v>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="X33" s="3" t="inlineStr">
         <is>
-          <t>At 28.0/100, Saif Ali Nagori stands out through modern python backend framework (fastapi/django), complemented by full stack capability (react/next.js/typescript). Plus embeddings-based retrieval system rounds out the build. Core evidence in Python, FastAPI, Flask, RAG, React maps to AI 7.0 and Python 17.0 bands. GitHub profile: GitHub API rate limit exceeded; skipped enrichment. Growth edge to probe in interview: low or dormant public github activity.</t>
+          <t>Saif Ali Nagori scored 38.0/100 (AI 7.0/40, Python 17.0/30, Cloud 4.0/15, GitHub 10.0/10), led by embeddings-based retrieval system and modern python backend framework (fastapi/django) Backed by full stack capability (react/next.js/typescript). Stack centers on Python, FastAPI, Flask, RAG. GitHub: Veteran Builder (3.1 yrs on GitHub, 26 repos [26 original], 102 contributions in past year [0 commits]). 10 relevant Python/AI repositories identified. Watch-item: limited redis or backend caching evidence. Fit for SDE AI internship is strong on shipped agentic depth.</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="X35" s="3" t="inlineStr">
         <is>
-          <t>Screening result: Agam Jain ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, FastAPI, PostgreSQL, Redis, Docker) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
+          <t>Agam, your portfolio demonstrates solid full-stack proficiency, particularly in building responsive interfaces with Next.js and managing state via React. However, we specifically require demonstrable experience with AI integration or agentic workflows to join this team. While your Python and FastAPI backend skills are strong, the absence of any RAG or LLM-driven project evidence means you haven’t met our core technical bar. To move forward, please highlight a specific project showcasing advanced AI implementation.</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="X40" s="3" t="inlineStr">
         <is>
-          <t>Screening result: Kartikay Sinha ineligible (0.0/100) — no evidence of python stack, no ai/agentic project evidence. Seen skills (Docker, React, Next.js, Typescript, Javascript) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
+          <t>Kartikay’s portfolio highlights a solid grasp of frontend engineering, particularly with React and Next.js. However, the role demands robust Python backend experience, which is entirely absent from your stack. More critically, we require demonstrable AI or agentic project evidence, such as RAG implementations, which you haven’t provided. To move forward, please prepare a Python-based project showcasing autonomous agent workflows. This specific technical depth is non-negotiable for this internship track.</t>
         </is>
       </c>
     </row>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="X47" s="3" t="inlineStr">
         <is>
-          <t>Shivam Raj does not advance (ineligible, 0.0/100). Core gap: no evidence of python stack, no ai/agentic project evidence. While Docker, Azure, React, Next.js, Typescript shows engineering interest, there is insufficient Python evidence and no production-grade agentic or retrieval pipeline. Successful candidates typically show async Python APIs wired to vector search, guardrailed agents, or evaluated RAG. Without that Python plus AI linkage, the profile falls below the hiring threshold.</t>
+          <t>Your portfolio highlights strong proficiency in modern frontend frameworks like Next.js and TypeScript, showcasing solid engineering fundamentals. However, we specifically require demonstrated backend expertise in Python, which is entirely absent from your experience. Furthermore, there is no evidence of AI or agentic system development, a core requirement for this role. To be considered, you must showcase projects involving Python-based backend services and concrete implementations of RAG or autonomous agent architectures.</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="X50" s="3" t="inlineStr">
         <is>
-          <t>Screening result: Vishwas Badiger ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Flask, React, Javascript, Node.Js) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
+          <t>Vishwas, your full-stack portfolio is solid, but the lack of AI integration is a hard stop. We specifically require evidence of agentic workflows or RAG implementation, which your Flask and React projects don't demonstrate. Your Python backend skills are a strong foundation, but they aren't enough on their own. To clear this bar, you need to showcase a project where you actively built or deployed an LLM-driven agent or retrieval system, not just standard CRUD operations.</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="X51" s="3" t="inlineStr">
         <is>
-          <t>Screening result: Yuvaraj R ineligible (0.0/100) — no ai/agentic project evidence. Seen skills (Python, Django, PostgreSQL, Docker, Rest Api) skew away from the required Python and AI/agentic core, with no convincing FastAPI/Django service or RAG/agent project to score. The internship requires demonstrable Python backend depth alongside LLM workflows, embeddings search, or multi-agent logic. Add a deployed Python + RAG/agent build to become competitive.</t>
+          <t>Your Django and PostgreSQL backend skills are solid, but we can’t move forward without concrete AI or agentic project evidence. The mandatory bar for this role requires demonstrated experience with RAG pipelines or autonomous agent frameworks, which your current portfolio lacks. To become competitive, build a distinct project showcasing LLM integration or agent orchestration. While your REST API and Docker experience shows good engineering fundamentals, the absence of AI-specific work prevents us from advancing your application further.</t>
         </is>
       </c>
     </row>

</xml_diff>